<commit_message>
Add 'PCRE2_UTF' option to PCRE2 and fix Feature Matrix.
</commit_message>
<xml_diff>
--- a/RegexFeatureMatrix.xlsx
+++ b/RegexFeatureMatrix.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Matrix" sheetId="1" r:id="R445d27dd1bcb490f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Matrix" sheetId="1" r:id="R6149067bec4440c4"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -71,7 +71,7 @@
   </x:si>
   <x:si>
     <x:t>Rust
- 1.98.0 </x:t>
+ 1.98.1 </x:t>
   </x:si>
   <x:si>
     <x:t>Java
@@ -17178,8 +17178,8 @@
       <x:c r="S57" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="T57" t="s">
-        <x:v>1</x:v>
+      <x:c r="T57" s="6" t="s">
+        <x:v>112</x:v>
       </x:c>
       <x:c r="U57" s="6" t="s">
         <x:v>112</x:v>
@@ -23994,8 +23994,8 @@
       <x:c r="S81" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="T81" t="s">
-        <x:v>1</x:v>
+      <x:c r="T81" s="6" t="s">
+        <x:v>112</x:v>
       </x:c>
       <x:c r="U81" s="6" t="s">
         <x:v>112</x:v>
@@ -62250,8 +62250,8 @@
       <x:c r="S219" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="T219" t="s">
-        <x:v>1</x:v>
+      <x:c r="T219" s="6" t="s">
+        <x:v>112</x:v>
       </x:c>
       <x:c r="U219" t="s">
         <x:v>1</x:v>

</xml_diff>

<commit_message>
Update PCRE2 engine: 10.48.
</commit_message>
<xml_diff>
--- a/RegexFeatureMatrix.xlsx
+++ b/RegexFeatureMatrix.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Matrix" sheetId="1" r:id="R6149067bec4440c4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Matrix" sheetId="1" r:id="Rd2f24b51688146ab"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -39,7 +39,7 @@
   </x:si>
   <x:si>
     <x:t>PCRE2
- 10.47 </x:t>
+ 10.48 </x:t>
   </x:si>
   <x:si>
     <x:t>Boost.Regex

</xml_diff>

<commit_message>
New Feature Matrix indicator: canonical equivalence of characters.
</commit_message>
<xml_diff>
--- a/RegexFeatureMatrix.xlsx
+++ b/RegexFeatureMatrix.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Matrix" sheetId="1" r:id="Rb3277afc90da4cb8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Matrix" sheetId="1" r:id="Reaa2dd3a460e4d19"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1335,7 +1335,13 @@
     <x:t>Miscellaneous</x:t>
   </x:si>
   <x:si>
+    <x:t>Captures</x:t>
+  </x:si>
+  <x:si>
     <x:t>Get all captures matched by group</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Empty≠Failed</x:t>
   </x:si>
   <x:si>
     <x:t>Differentiate between empty groups and failed groups</x:t>
@@ -1405,6 +1411,12 @@
   </x:si>
   <x:si>
     <x:t>Support Unicode case folding</x:t>
+  </x:si>
+  <x:si>
+    <x:t>é=e+´</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Canonical equivalence of characters</x:t>
   </x:si>
   <x:si>
     <x:t>Σσς</x:t>
@@ -1477,6 +1489,9 @@
   </x:si>
   <x:si>
     <x:t>Complement (pattern must not match)</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Alt. syntax</x:t>
   </x:si>
   <x:si>
     <x:t>Support alternative syntax</x:t>
@@ -60687,10 +60702,10 @@
     </x:row>
     <x:row r="208">
       <x:c r="A208" s="4" t="s">
-        <x:v>1</x:v>
+        <x:v>432</x:v>
       </x:c>
       <x:c r="B208" s="5" t="s">
-        <x:v>432</x:v>
+        <x:v>433</x:v>
       </x:c>
       <x:c r="C208" s="6" t="s">
         <x:v>115</x:v>
@@ -60992,10 +61007,10 @@
     </x:row>
     <x:row r="209">
       <x:c r="A209" s="4" t="s">
-        <x:v>1</x:v>
+        <x:v>434</x:v>
       </x:c>
       <x:c r="B209" s="5" t="s">
-        <x:v>433</x:v>
+        <x:v>435</x:v>
       </x:c>
       <x:c r="C209" s="6" t="s">
         <x:v>115</x:v>
@@ -61297,10 +61312,10 @@
     </x:row>
     <x:row r="210">
       <x:c r="A210" s="4" t="s">
-        <x:v>434</x:v>
+        <x:v>436</x:v>
       </x:c>
       <x:c r="B210" s="5" t="s">
-        <x:v>435</x:v>
+        <x:v>437</x:v>
       </x:c>
       <x:c r="C210" t="s">
         <x:v>1</x:v>
@@ -61602,10 +61617,10 @@
     </x:row>
     <x:row r="211">
       <x:c r="A211" s="4" t="s">
-        <x:v>436</x:v>
+        <x:v>438</x:v>
       </x:c>
       <x:c r="B211" s="5" t="s">
-        <x:v>437</x:v>
+        <x:v>439</x:v>
       </x:c>
       <x:c r="C211" t="s">
         <x:v>1</x:v>
@@ -61907,10 +61922,10 @@
     </x:row>
     <x:row r="212">
       <x:c r="A212" s="4" t="s">
-        <x:v>438</x:v>
+        <x:v>440</x:v>
       </x:c>
       <x:c r="B212" s="5" t="s">
-        <x:v>439</x:v>
+        <x:v>441</x:v>
       </x:c>
       <x:c r="C212" t="s">
         <x:v>1</x:v>
@@ -62212,10 +62227,10 @@
     </x:row>
     <x:row r="213">
       <x:c r="A213" s="4" t="s">
-        <x:v>440</x:v>
+        <x:v>442</x:v>
       </x:c>
       <x:c r="B213" s="5" t="s">
-        <x:v>441</x:v>
+        <x:v>443</x:v>
       </x:c>
       <x:c r="C213" t="s">
         <x:v>1</x:v>
@@ -62517,10 +62532,10 @@
     </x:row>
     <x:row r="214">
       <x:c r="A214" s="4" t="s">
-        <x:v>442</x:v>
+        <x:v>444</x:v>
       </x:c>
       <x:c r="B214" s="5" t="s">
-        <x:v>443</x:v>
+        <x:v>445</x:v>
       </x:c>
       <x:c r="C214" t="s">
         <x:v>1</x:v>
@@ -62822,10 +62837,10 @@
     </x:row>
     <x:row r="215">
       <x:c r="A215" s="4" t="s">
-        <x:v>444</x:v>
+        <x:v>446</x:v>
       </x:c>
       <x:c r="B215" s="5" t="s">
-        <x:v>445</x:v>
+        <x:v>447</x:v>
       </x:c>
       <x:c r="C215" t="s">
         <x:v>1</x:v>
@@ -63127,10 +63142,10 @@
     </x:row>
     <x:row r="216">
       <x:c r="A216" s="4" t="s">
-        <x:v>446</x:v>
+        <x:v>448</x:v>
       </x:c>
       <x:c r="B216" s="5" t="s">
-        <x:v>447</x:v>
+        <x:v>449</x:v>
       </x:c>
       <x:c r="C216" s="6" t="s">
         <x:v>115</x:v>
@@ -63432,10 +63447,10 @@
     </x:row>
     <x:row r="217">
       <x:c r="A217" s="4" t="s">
-        <x:v>448</x:v>
+        <x:v>450</x:v>
       </x:c>
       <x:c r="B217" s="5" t="s">
-        <x:v>449</x:v>
+        <x:v>451</x:v>
       </x:c>
       <x:c r="C217" s="6" t="s">
         <x:v>115</x:v>
@@ -63737,10 +63752,10 @@
     </x:row>
     <x:row r="218">
       <x:c r="A218" s="4" t="s">
-        <x:v>450</x:v>
+        <x:v>452</x:v>
       </x:c>
       <x:c r="B218" s="5" t="s">
-        <x:v>451</x:v>
+        <x:v>453</x:v>
       </x:c>
       <x:c r="C218" s="6" t="s">
         <x:v>115</x:v>
@@ -64042,10 +64057,10 @@
     </x:row>
     <x:row r="219">
       <x:c r="A219" s="4" t="s">
-        <x:v>452</x:v>
+        <x:v>454</x:v>
       </x:c>
       <x:c r="B219" s="5" t="s">
-        <x:v>453</x:v>
+        <x:v>455</x:v>
       </x:c>
       <x:c r="C219" t="s">
         <x:v>1</x:v>
@@ -64347,10 +64362,10 @@
     </x:row>
     <x:row r="220">
       <x:c r="A220" s="4" t="s">
-        <x:v>454</x:v>
+        <x:v>456</x:v>
       </x:c>
       <x:c r="B220" s="5" t="s">
-        <x:v>455</x:v>
+        <x:v>457</x:v>
       </x:c>
       <x:c r="C220" s="6" t="s">
         <x:v>115</x:v>
@@ -64652,10 +64667,10 @@
     </x:row>
     <x:row r="221">
       <x:c r="A221" s="4" t="s">
-        <x:v>456</x:v>
+        <x:v>458</x:v>
       </x:c>
       <x:c r="B221" s="5" t="s">
-        <x:v>457</x:v>
+        <x:v>459</x:v>
       </x:c>
       <x:c r="C221" t="s">
         <x:v>1</x:v>
@@ -64663,8 +64678,8 @@
       <x:c r="D221" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="E221" s="6" t="s">
-        <x:v>115</x:v>
+      <x:c r="E221" t="s">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="F221" t="s">
         <x:v>1</x:v>
@@ -64690,26 +64705,26 @@
       <x:c r="M221" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="N221" s="6" t="s">
-        <x:v>115</x:v>
-      </x:c>
-      <x:c r="O221" s="6" t="s">
-        <x:v>115</x:v>
-      </x:c>
-      <x:c r="P221" s="6" t="s">
-        <x:v>115</x:v>
-      </x:c>
-      <x:c r="Q221" s="6" t="s">
-        <x:v>115</x:v>
-      </x:c>
-      <x:c r="R221" s="6" t="s">
-        <x:v>115</x:v>
+      <x:c r="N221" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="O221" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P221" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="Q221" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="R221" t="s">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="S221" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="T221" s="6" t="s">
-        <x:v>115</x:v>
+      <x:c r="T221" t="s">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="U221" t="s">
         <x:v>1</x:v>
@@ -64738,98 +64753,98 @@
       <x:c r="AC221" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="AD221" s="6" t="s">
-        <x:v>115</x:v>
-      </x:c>
-      <x:c r="AE221" s="6" t="s">
-        <x:v>115</x:v>
-      </x:c>
-      <x:c r="AF221" s="6" t="s">
-        <x:v>115</x:v>
-      </x:c>
-      <x:c r="AG221" s="6" t="s">
-        <x:v>115</x:v>
-      </x:c>
-      <x:c r="AH221" s="6" t="s">
-        <x:v>115</x:v>
-      </x:c>
-      <x:c r="AI221" s="6" t="s">
-        <x:v>115</x:v>
-      </x:c>
-      <x:c r="AJ221" s="6" t="s">
-        <x:v>115</x:v>
-      </x:c>
-      <x:c r="AK221" s="6" t="s">
-        <x:v>115</x:v>
-      </x:c>
-      <x:c r="AL221" s="6" t="s">
-        <x:v>115</x:v>
-      </x:c>
-      <x:c r="AM221" s="6" t="s">
-        <x:v>115</x:v>
-      </x:c>
-      <x:c r="AN221" s="6" t="s">
-        <x:v>115</x:v>
-      </x:c>
-      <x:c r="AO221" s="6" t="s">
-        <x:v>115</x:v>
-      </x:c>
-      <x:c r="AP221" s="6" t="s">
-        <x:v>115</x:v>
-      </x:c>
-      <x:c r="AQ221" s="6" t="s">
-        <x:v>115</x:v>
-      </x:c>
-      <x:c r="AR221" s="6" t="s">
-        <x:v>115</x:v>
-      </x:c>
-      <x:c r="AS221" s="6" t="s">
-        <x:v>115</x:v>
-      </x:c>
-      <x:c r="AT221" s="6" t="s">
-        <x:v>115</x:v>
-      </x:c>
-      <x:c r="AU221" s="6" t="s">
-        <x:v>115</x:v>
+      <x:c r="AD221" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AE221" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AF221" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AG221" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AH221" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AI221" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AJ221" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AK221" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AL221" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AM221" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AN221" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AO221" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AP221" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AQ221" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AR221" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AS221" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AT221" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AU221" t="s">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="AV221" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="AW221" s="6" t="s">
-        <x:v>115</x:v>
-      </x:c>
-      <x:c r="AX221" s="6" t="s">
-        <x:v>115</x:v>
-      </x:c>
-      <x:c r="AY221" s="6" t="s">
-        <x:v>115</x:v>
-      </x:c>
-      <x:c r="AZ221" s="6" t="s">
-        <x:v>115</x:v>
+      <x:c r="AW221" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AX221" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AY221" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AZ221" t="s">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="BA221" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="BB221" s="6" t="s">
-        <x:v>115</x:v>
-      </x:c>
-      <x:c r="BC221" s="6" t="s">
-        <x:v>115</x:v>
-      </x:c>
-      <x:c r="BD221" s="6" t="s">
-        <x:v>115</x:v>
+      <x:c r="BB221" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BC221" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BD221" t="s">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="BE221" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="BF221" s="6" t="s">
-        <x:v>115</x:v>
-      </x:c>
-      <x:c r="BG221" s="6" t="s">
-        <x:v>115</x:v>
-      </x:c>
-      <x:c r="BH221" s="6" t="s">
-        <x:v>115</x:v>
+      <x:c r="BF221" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BG221" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BH221" t="s">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="BI221" t="s">
         <x:v>1</x:v>
@@ -64837,41 +64852,41 @@
       <x:c r="BJ221" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="BK221" s="6" t="s">
-        <x:v>115</x:v>
+      <x:c r="BK221" t="s">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="BL221" s="6" t="s">
         <x:v>115</x:v>
       </x:c>
-      <x:c r="BM221" s="6" t="s">
-        <x:v>115</x:v>
-      </x:c>
-      <x:c r="BN221" s="6" t="s">
-        <x:v>115</x:v>
+      <x:c r="BM221" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BN221" t="s">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="BO221" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="BP221" s="6" t="s">
-        <x:v>115</x:v>
-      </x:c>
-      <x:c r="BQ221" s="6" t="s">
-        <x:v>115</x:v>
-      </x:c>
-      <x:c r="BR221" s="6" t="s">
-        <x:v>115</x:v>
-      </x:c>
-      <x:c r="BS221" s="6" t="s">
-        <x:v>115</x:v>
-      </x:c>
-      <x:c r="BT221" s="6" t="s">
-        <x:v>115</x:v>
-      </x:c>
-      <x:c r="BU221" s="6" t="s">
-        <x:v>115</x:v>
-      </x:c>
-      <x:c r="BV221" s="6" t="s">
-        <x:v>115</x:v>
+      <x:c r="BP221" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BQ221" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BR221" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BS221" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BT221" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BU221" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BV221" t="s">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="BW221" t="s">
         <x:v>1</x:v>
@@ -64894,11 +64909,11 @@
       <x:c r="CC221" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="CD221" s="6" t="s">
-        <x:v>115</x:v>
-      </x:c>
-      <x:c r="CE221" s="6" t="s">
-        <x:v>115</x:v>
+      <x:c r="CD221" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="CE221" t="s">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="CF221" t="s">
         <x:v>1</x:v>
@@ -64915,52 +64930,52 @@
       <x:c r="CJ221" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="CK221" s="6" t="s">
-        <x:v>115</x:v>
-      </x:c>
-      <x:c r="CL221" s="6" t="s">
-        <x:v>115</x:v>
-      </x:c>
-      <x:c r="CM221" s="6" t="s">
-        <x:v>115</x:v>
+      <x:c r="CK221" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="CL221" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="CM221" t="s">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="CN221" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="CO221" s="6" t="s">
-        <x:v>115</x:v>
+      <x:c r="CO221" t="s">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="CP221" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="CQ221" s="6" t="s">
-        <x:v>115</x:v>
-      </x:c>
-      <x:c r="CR221" s="6" t="s">
-        <x:v>115</x:v>
-      </x:c>
-      <x:c r="CS221" s="6" t="s">
-        <x:v>115</x:v>
-      </x:c>
-      <x:c r="CT221" s="6" t="s">
-        <x:v>115</x:v>
-      </x:c>
-      <x:c r="CU221" s="6" t="s">
-        <x:v>115</x:v>
+      <x:c r="CQ221" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="CR221" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="CS221" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="CT221" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="CU221" t="s">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="CV221" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="CW221" s="6" t="s">
-        <x:v>115</x:v>
+      <x:c r="CW221" t="s">
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="222">
       <x:c r="A222" s="4" t="s">
-        <x:v>458</x:v>
+        <x:v>460</x:v>
       </x:c>
       <x:c r="B222" s="5" t="s">
-        <x:v>459</x:v>
+        <x:v>461</x:v>
       </x:c>
       <x:c r="C222" t="s">
         <x:v>1</x:v>
@@ -64968,8 +64983,8 @@
       <x:c r="D222" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="E222" t="s">
-        <x:v>1</x:v>
+      <x:c r="E222" s="6" t="s">
+        <x:v>115</x:v>
       </x:c>
       <x:c r="F222" t="s">
         <x:v>1</x:v>
@@ -64995,26 +65010,26 @@
       <x:c r="M222" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="N222" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="O222" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="P222" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="Q222" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="R222" t="s">
-        <x:v>1</x:v>
+      <x:c r="N222" s="6" t="s">
+        <x:v>115</x:v>
+      </x:c>
+      <x:c r="O222" s="6" t="s">
+        <x:v>115</x:v>
+      </x:c>
+      <x:c r="P222" s="6" t="s">
+        <x:v>115</x:v>
+      </x:c>
+      <x:c r="Q222" s="6" t="s">
+        <x:v>115</x:v>
+      </x:c>
+      <x:c r="R222" s="6" t="s">
+        <x:v>115</x:v>
       </x:c>
       <x:c r="S222" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="T222" t="s">
-        <x:v>1</x:v>
+      <x:c r="T222" s="6" t="s">
+        <x:v>115</x:v>
       </x:c>
       <x:c r="U222" t="s">
         <x:v>1</x:v>
@@ -65076,65 +65091,65 @@
       <x:c r="AN222" s="6" t="s">
         <x:v>115</x:v>
       </x:c>
-      <x:c r="AO222" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AP222" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AQ222" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AR222" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AS222" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AT222" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AU222" t="s">
-        <x:v>1</x:v>
+      <x:c r="AO222" s="6" t="s">
+        <x:v>115</x:v>
+      </x:c>
+      <x:c r="AP222" s="6" t="s">
+        <x:v>115</x:v>
+      </x:c>
+      <x:c r="AQ222" s="6" t="s">
+        <x:v>115</x:v>
+      </x:c>
+      <x:c r="AR222" s="6" t="s">
+        <x:v>115</x:v>
+      </x:c>
+      <x:c r="AS222" s="6" t="s">
+        <x:v>115</x:v>
+      </x:c>
+      <x:c r="AT222" s="6" t="s">
+        <x:v>115</x:v>
+      </x:c>
+      <x:c r="AU222" s="6" t="s">
+        <x:v>115</x:v>
       </x:c>
       <x:c r="AV222" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="AW222" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AX222" t="s">
-        <x:v>1</x:v>
+      <x:c r="AW222" s="6" t="s">
+        <x:v>115</x:v>
+      </x:c>
+      <x:c r="AX222" s="6" t="s">
+        <x:v>115</x:v>
       </x:c>
       <x:c r="AY222" s="6" t="s">
         <x:v>115</x:v>
       </x:c>
-      <x:c r="AZ222" t="s">
-        <x:v>1</x:v>
+      <x:c r="AZ222" s="6" t="s">
+        <x:v>115</x:v>
       </x:c>
       <x:c r="BA222" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="BB222" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BC222" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BD222" t="s">
-        <x:v>1</x:v>
+      <x:c r="BB222" s="6" t="s">
+        <x:v>115</x:v>
+      </x:c>
+      <x:c r="BC222" s="6" t="s">
+        <x:v>115</x:v>
+      </x:c>
+      <x:c r="BD222" s="6" t="s">
+        <x:v>115</x:v>
       </x:c>
       <x:c r="BE222" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="BF222" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BG222" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BH222" t="s">
-        <x:v>1</x:v>
+      <x:c r="BF222" s="6" t="s">
+        <x:v>115</x:v>
+      </x:c>
+      <x:c r="BG222" s="6" t="s">
+        <x:v>115</x:v>
+      </x:c>
+      <x:c r="BH222" s="6" t="s">
+        <x:v>115</x:v>
       </x:c>
       <x:c r="BI222" t="s">
         <x:v>1</x:v>
@@ -65145,14 +65160,14 @@
       <x:c r="BK222" s="6" t="s">
         <x:v>115</x:v>
       </x:c>
-      <x:c r="BL222" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BM222" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BN222" t="s">
-        <x:v>1</x:v>
+      <x:c r="BL222" s="6" t="s">
+        <x:v>115</x:v>
+      </x:c>
+      <x:c r="BM222" s="6" t="s">
+        <x:v>115</x:v>
+      </x:c>
+      <x:c r="BN222" s="6" t="s">
+        <x:v>115</x:v>
       </x:c>
       <x:c r="BO222" t="s">
         <x:v>1</x:v>
@@ -65160,8 +65175,8 @@
       <x:c r="BP222" s="6" t="s">
         <x:v>115</x:v>
       </x:c>
-      <x:c r="BQ222" t="s">
-        <x:v>1</x:v>
+      <x:c r="BQ222" s="6" t="s">
+        <x:v>115</x:v>
       </x:c>
       <x:c r="BR222" s="6" t="s">
         <x:v>115</x:v>
@@ -65169,11 +65184,11 @@
       <x:c r="BS222" s="6" t="s">
         <x:v>115</x:v>
       </x:c>
-      <x:c r="BT222" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BU222" t="s">
-        <x:v>1</x:v>
+      <x:c r="BT222" s="6" t="s">
+        <x:v>115</x:v>
+      </x:c>
+      <x:c r="BU222" s="6" t="s">
+        <x:v>115</x:v>
       </x:c>
       <x:c r="BV222" s="6" t="s">
         <x:v>115</x:v>
@@ -65199,11 +65214,11 @@
       <x:c r="CC222" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="CD222" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="CE222" t="s">
-        <x:v>1</x:v>
+      <x:c r="CD222" s="6" t="s">
+        <x:v>115</x:v>
+      </x:c>
+      <x:c r="CE222" s="6" t="s">
+        <x:v>115</x:v>
       </x:c>
       <x:c r="CF222" t="s">
         <x:v>1</x:v>
@@ -65223,32 +65238,32 @@
       <x:c r="CK222" s="6" t="s">
         <x:v>115</x:v>
       </x:c>
-      <x:c r="CL222" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="CM222" t="s">
-        <x:v>1</x:v>
+      <x:c r="CL222" s="6" t="s">
+        <x:v>115</x:v>
+      </x:c>
+      <x:c r="CM222" s="6" t="s">
+        <x:v>115</x:v>
       </x:c>
       <x:c r="CN222" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="CO222" t="s">
-        <x:v>1</x:v>
+      <x:c r="CO222" s="6" t="s">
+        <x:v>115</x:v>
       </x:c>
       <x:c r="CP222" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="CQ222" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="CR222" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="CS222" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="CT222" t="s">
-        <x:v>1</x:v>
+      <x:c r="CQ222" s="6" t="s">
+        <x:v>115</x:v>
+      </x:c>
+      <x:c r="CR222" s="6" t="s">
+        <x:v>115</x:v>
+      </x:c>
+      <x:c r="CS222" s="6" t="s">
+        <x:v>115</x:v>
+      </x:c>
+      <x:c r="CT222" s="6" t="s">
+        <x:v>115</x:v>
       </x:c>
       <x:c r="CU222" s="6" t="s">
         <x:v>115</x:v>
@@ -65256,16 +65271,16 @@
       <x:c r="CV222" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="CW222" t="s">
-        <x:v>1</x:v>
+      <x:c r="CW222" s="6" t="s">
+        <x:v>115</x:v>
       </x:c>
     </x:row>
     <x:row r="223">
       <x:c r="A223" s="4" t="s">
-        <x:v>460</x:v>
+        <x:v>462</x:v>
       </x:c>
       <x:c r="B223" s="5" t="s">
-        <x:v>461</x:v>
+        <x:v>463</x:v>
       </x:c>
       <x:c r="C223" t="s">
         <x:v>1</x:v>
@@ -65348,38 +65363,38 @@
       <x:c r="AC223" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="AD223" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AE223" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AF223" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AG223" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AH223" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AI223" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AJ223" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AK223" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AL223" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AM223" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AN223" t="s">
-        <x:v>1</x:v>
+      <x:c r="AD223" s="6" t="s">
+        <x:v>115</x:v>
+      </x:c>
+      <x:c r="AE223" s="6" t="s">
+        <x:v>115</x:v>
+      </x:c>
+      <x:c r="AF223" s="6" t="s">
+        <x:v>115</x:v>
+      </x:c>
+      <x:c r="AG223" s="6" t="s">
+        <x:v>115</x:v>
+      </x:c>
+      <x:c r="AH223" s="6" t="s">
+        <x:v>115</x:v>
+      </x:c>
+      <x:c r="AI223" s="6" t="s">
+        <x:v>115</x:v>
+      </x:c>
+      <x:c r="AJ223" s="6" t="s">
+        <x:v>115</x:v>
+      </x:c>
+      <x:c r="AK223" s="6" t="s">
+        <x:v>115</x:v>
+      </x:c>
+      <x:c r="AL223" s="6" t="s">
+        <x:v>115</x:v>
+      </x:c>
+      <x:c r="AM223" s="6" t="s">
+        <x:v>115</x:v>
+      </x:c>
+      <x:c r="AN223" s="6" t="s">
+        <x:v>115</x:v>
       </x:c>
       <x:c r="AO223" t="s">
         <x:v>1</x:v>
@@ -65405,14 +65420,14 @@
       <x:c r="AV223" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="AW223" s="6" t="s">
-        <x:v>115</x:v>
+      <x:c r="AW223" t="s">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="AX223" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="AY223" t="s">
-        <x:v>1</x:v>
+      <x:c r="AY223" s="6" t="s">
+        <x:v>115</x:v>
       </x:c>
       <x:c r="AZ223" t="s">
         <x:v>1</x:v>
@@ -65447,8 +65462,8 @@
       <x:c r="BJ223" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="BK223" t="s">
-        <x:v>1</x:v>
+      <x:c r="BK223" s="6" t="s">
+        <x:v>115</x:v>
       </x:c>
       <x:c r="BL223" t="s">
         <x:v>1</x:v>
@@ -65462,8 +65477,8 @@
       <x:c r="BO223" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="BP223" t="s">
-        <x:v>1</x:v>
+      <x:c r="BP223" s="6" t="s">
+        <x:v>115</x:v>
       </x:c>
       <x:c r="BQ223" t="s">
         <x:v>1</x:v>
@@ -65480,8 +65495,8 @@
       <x:c r="BU223" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="BV223" t="s">
-        <x:v>1</x:v>
+      <x:c r="BV223" s="6" t="s">
+        <x:v>115</x:v>
       </x:c>
       <x:c r="BW223" t="s">
         <x:v>1</x:v>
@@ -65492,11 +65507,11 @@
       <x:c r="BY223" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="BZ223" s="6" t="s">
-        <x:v>115</x:v>
-      </x:c>
-      <x:c r="CA223" s="6" t="s">
-        <x:v>115</x:v>
+      <x:c r="BZ223" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="CA223" t="s">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="CB223" t="s">
         <x:v>1</x:v>
@@ -65525,8 +65540,8 @@
       <x:c r="CJ223" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="CK223" t="s">
-        <x:v>1</x:v>
+      <x:c r="CK223" s="6" t="s">
+        <x:v>115</x:v>
       </x:c>
       <x:c r="CL223" t="s">
         <x:v>1</x:v>
@@ -65555,8 +65570,8 @@
       <x:c r="CT223" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="CU223" t="s">
-        <x:v>1</x:v>
+      <x:c r="CU223" s="6" t="s">
+        <x:v>115</x:v>
       </x:c>
       <x:c r="CV223" t="s">
         <x:v>1</x:v>
@@ -65567,19 +65582,19 @@
     </x:row>
     <x:row r="224">
       <x:c r="A224" s="4" t="s">
-        <x:v>462</x:v>
+        <x:v>464</x:v>
       </x:c>
       <x:c r="B224" s="5" t="s">
-        <x:v>463</x:v>
+        <x:v>465</x:v>
       </x:c>
       <x:c r="C224" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="D224" s="6" t="s">
-        <x:v>115</x:v>
-      </x:c>
-      <x:c r="E224" s="6" t="s">
-        <x:v>115</x:v>
+      <x:c r="D224" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E224" t="s">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="F224" t="s">
         <x:v>1</x:v>
@@ -65611,20 +65626,20 @@
       <x:c r="O224" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="P224" s="6" t="s">
-        <x:v>115</x:v>
-      </x:c>
-      <x:c r="Q224" s="6" t="s">
-        <x:v>115</x:v>
-      </x:c>
-      <x:c r="R224" s="6" t="s">
-        <x:v>115</x:v>
+      <x:c r="P224" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="Q224" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="R224" t="s">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="S224" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="T224" s="6" t="s">
-        <x:v>115</x:v>
+      <x:c r="T224" t="s">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="U224" t="s">
         <x:v>1</x:v>
@@ -65653,38 +65668,38 @@
       <x:c r="AC224" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="AD224" s="6" t="s">
-        <x:v>115</x:v>
-      </x:c>
-      <x:c r="AE224" s="6" t="s">
-        <x:v>115</x:v>
-      </x:c>
-      <x:c r="AF224" s="6" t="s">
-        <x:v>115</x:v>
-      </x:c>
-      <x:c r="AG224" s="6" t="s">
-        <x:v>115</x:v>
-      </x:c>
-      <x:c r="AH224" s="6" t="s">
-        <x:v>115</x:v>
-      </x:c>
-      <x:c r="AI224" s="6" t="s">
-        <x:v>115</x:v>
-      </x:c>
-      <x:c r="AJ224" s="6" t="s">
-        <x:v>115</x:v>
-      </x:c>
-      <x:c r="AK224" s="6" t="s">
-        <x:v>115</x:v>
-      </x:c>
-      <x:c r="AL224" s="6" t="s">
-        <x:v>115</x:v>
-      </x:c>
-      <x:c r="AM224" s="6" t="s">
-        <x:v>115</x:v>
-      </x:c>
-      <x:c r="AN224" s="6" t="s">
-        <x:v>115</x:v>
+      <x:c r="AD224" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AE224" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AF224" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AG224" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AH224" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AI224" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AJ224" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AK224" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AL224" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AM224" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AN224" t="s">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="AO224" t="s">
         <x:v>1</x:v>
@@ -65698,11 +65713,11 @@
       <x:c r="AR224" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="AS224" s="6" t="s">
-        <x:v>115</x:v>
-      </x:c>
-      <x:c r="AT224" s="6" t="s">
-        <x:v>115</x:v>
+      <x:c r="AS224" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AT224" t="s">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="AU224" t="s">
         <x:v>1</x:v>
@@ -65713,62 +65728,62 @@
       <x:c r="AW224" s="6" t="s">
         <x:v>115</x:v>
       </x:c>
-      <x:c r="AX224" s="6" t="s">
-        <x:v>115</x:v>
+      <x:c r="AX224" t="s">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="AY224" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="AZ224" s="6" t="s">
-        <x:v>115</x:v>
-      </x:c>
-      <x:c r="BA224" s="6" t="s">
-        <x:v>115</x:v>
-      </x:c>
-      <x:c r="BB224" s="6" t="s">
-        <x:v>115</x:v>
+      <x:c r="AZ224" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BA224" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BB224" t="s">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="BC224" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="BD224" s="6" t="s">
-        <x:v>115</x:v>
+      <x:c r="BD224" t="s">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="BE224" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="BF224" s="6" t="s">
-        <x:v>115</x:v>
-      </x:c>
-      <x:c r="BG224" s="6" t="s">
-        <x:v>115</x:v>
-      </x:c>
-      <x:c r="BH224" s="6" t="s">
-        <x:v>115</x:v>
+      <x:c r="BF224" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BG224" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BH224" t="s">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="BI224" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="BJ224" s="6" t="s">
-        <x:v>115</x:v>
-      </x:c>
-      <x:c r="BK224" s="6" t="s">
-        <x:v>115</x:v>
-      </x:c>
-      <x:c r="BL224" s="6" t="s">
-        <x:v>115</x:v>
-      </x:c>
-      <x:c r="BM224" s="6" t="s">
-        <x:v>115</x:v>
-      </x:c>
-      <x:c r="BN224" s="6" t="s">
-        <x:v>115</x:v>
-      </x:c>
-      <x:c r="BO224" s="6" t="s">
-        <x:v>115</x:v>
-      </x:c>
-      <x:c r="BP224" s="6" t="s">
-        <x:v>115</x:v>
+      <x:c r="BJ224" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BK224" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BL224" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BM224" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BN224" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BO224" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BP224" t="s">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="BQ224" t="s">
         <x:v>1</x:v>
@@ -65779,23 +65794,23 @@
       <x:c r="BS224" s="6" t="s">
         <x:v>115</x:v>
       </x:c>
-      <x:c r="BT224" s="6" t="s">
-        <x:v>115</x:v>
-      </x:c>
-      <x:c r="BU224" s="6" t="s">
-        <x:v>115</x:v>
-      </x:c>
-      <x:c r="BV224" s="6" t="s">
-        <x:v>115</x:v>
-      </x:c>
-      <x:c r="BW224" s="6" t="s">
-        <x:v>115</x:v>
+      <x:c r="BT224" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BU224" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BV224" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BW224" t="s">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="BX224" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="BY224" s="6" t="s">
-        <x:v>115</x:v>
+      <x:c r="BY224" t="s">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="BZ224" s="6" t="s">
         <x:v>115</x:v>
@@ -65803,20 +65818,20 @@
       <x:c r="CA224" s="6" t="s">
         <x:v>115</x:v>
       </x:c>
-      <x:c r="CB224" s="6" t="s">
-        <x:v>115</x:v>
+      <x:c r="CB224" t="s">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="CC224" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="CD224" s="6" t="s">
-        <x:v>115</x:v>
-      </x:c>
-      <x:c r="CE224" s="6" t="s">
-        <x:v>115</x:v>
-      </x:c>
-      <x:c r="CF224" s="6" t="s">
-        <x:v>115</x:v>
+      <x:c r="CD224" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="CE224" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="CF224" t="s">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="CG224" t="s">
         <x:v>1</x:v>
@@ -65824,35 +65839,35 @@
       <x:c r="CH224" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="CI224" s="6" t="s">
-        <x:v>115</x:v>
-      </x:c>
-      <x:c r="CJ224" s="6" t="s">
-        <x:v>115</x:v>
-      </x:c>
-      <x:c r="CK224" s="6" t="s">
-        <x:v>115</x:v>
-      </x:c>
-      <x:c r="CL224" s="6" t="s">
-        <x:v>115</x:v>
-      </x:c>
-      <x:c r="CM224" s="6" t="s">
-        <x:v>115</x:v>
-      </x:c>
-      <x:c r="CN224" s="6" t="s">
-        <x:v>115</x:v>
+      <x:c r="CI224" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="CJ224" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="CK224" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="CL224" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="CM224" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="CN224" t="s">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="CO224" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="CP224" s="6" t="s">
-        <x:v>115</x:v>
-      </x:c>
-      <x:c r="CQ224" s="6" t="s">
-        <x:v>115</x:v>
-      </x:c>
-      <x:c r="CR224" s="6" t="s">
-        <x:v>115</x:v>
+      <x:c r="CP224" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="CQ224" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="CR224" t="s">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="CS224" t="s">
         <x:v>1</x:v>
@@ -65860,136 +65875,136 @@
       <x:c r="CT224" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="CU224" s="6" t="s">
-        <x:v>115</x:v>
-      </x:c>
-      <x:c r="CV224" s="6" t="s">
-        <x:v>115</x:v>
-      </x:c>
-      <x:c r="CW224" s="6" t="s">
-        <x:v>115</x:v>
+      <x:c r="CU224" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="CV224" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="CW224" t="s">
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="225">
       <x:c r="A225" s="4" t="s">
-        <x:v>464</x:v>
+        <x:v>466</x:v>
       </x:c>
       <x:c r="B225" s="5" t="s">
-        <x:v>465</x:v>
+        <x:v>467</x:v>
       </x:c>
       <x:c r="C225" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="D225" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E225" t="s">
-        <x:v>1</x:v>
+      <x:c r="D225" s="6" t="s">
+        <x:v>115</x:v>
+      </x:c>
+      <x:c r="E225" s="6" t="s">
+        <x:v>115</x:v>
       </x:c>
       <x:c r="F225" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="G225" s="6" t="s">
-        <x:v>115</x:v>
-      </x:c>
-      <x:c r="H225" s="6" t="s">
-        <x:v>115</x:v>
-      </x:c>
-      <x:c r="I225" s="6" t="s">
-        <x:v>115</x:v>
-      </x:c>
-      <x:c r="J225" s="6" t="s">
-        <x:v>115</x:v>
-      </x:c>
-      <x:c r="K225" s="6" t="s">
-        <x:v>115</x:v>
-      </x:c>
-      <x:c r="L225" s="6" t="s">
-        <x:v>115</x:v>
+      <x:c r="G225" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H225" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="I225" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J225" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="K225" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="L225" t="s">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="M225" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="N225" s="6" t="s">
-        <x:v>115</x:v>
-      </x:c>
-      <x:c r="O225" s="6" t="s">
-        <x:v>115</x:v>
-      </x:c>
-      <x:c r="P225" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="Q225" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="R225" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="S225" s="6" t="s">
-        <x:v>115</x:v>
-      </x:c>
-      <x:c r="T225" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="U225" s="6" t="s">
-        <x:v>115</x:v>
-      </x:c>
-      <x:c r="V225" s="6" t="s">
-        <x:v>115</x:v>
-      </x:c>
-      <x:c r="W225" s="6" t="s">
-        <x:v>115</x:v>
-      </x:c>
-      <x:c r="X225" s="6" t="s">
-        <x:v>115</x:v>
-      </x:c>
-      <x:c r="Y225" s="6" t="s">
-        <x:v>115</x:v>
-      </x:c>
-      <x:c r="Z225" s="6" t="s">
-        <x:v>115</x:v>
-      </x:c>
-      <x:c r="AA225" s="6" t="s">
-        <x:v>115</x:v>
-      </x:c>
-      <x:c r="AB225" s="6" t="s">
-        <x:v>115</x:v>
-      </x:c>
-      <x:c r="AC225" s="6" t="s">
-        <x:v>115</x:v>
-      </x:c>
-      <x:c r="AD225" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AE225" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AF225" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AG225" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AH225" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AI225" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AJ225" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AK225" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AL225" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AM225" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AN225" t="s">
-        <x:v>1</x:v>
+      <x:c r="N225" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="O225" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P225" s="6" t="s">
+        <x:v>115</x:v>
+      </x:c>
+      <x:c r="Q225" s="6" t="s">
+        <x:v>115</x:v>
+      </x:c>
+      <x:c r="R225" s="6" t="s">
+        <x:v>115</x:v>
+      </x:c>
+      <x:c r="S225" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="T225" s="6" t="s">
+        <x:v>115</x:v>
+      </x:c>
+      <x:c r="U225" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="V225" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="W225" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="X225" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="Y225" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="Z225" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AA225" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AB225" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AC225" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AD225" s="6" t="s">
+        <x:v>115</x:v>
+      </x:c>
+      <x:c r="AE225" s="6" t="s">
+        <x:v>115</x:v>
+      </x:c>
+      <x:c r="AF225" s="6" t="s">
+        <x:v>115</x:v>
+      </x:c>
+      <x:c r="AG225" s="6" t="s">
+        <x:v>115</x:v>
+      </x:c>
+      <x:c r="AH225" s="6" t="s">
+        <x:v>115</x:v>
+      </x:c>
+      <x:c r="AI225" s="6" t="s">
+        <x:v>115</x:v>
+      </x:c>
+      <x:c r="AJ225" s="6" t="s">
+        <x:v>115</x:v>
+      </x:c>
+      <x:c r="AK225" s="6" t="s">
+        <x:v>115</x:v>
+      </x:c>
+      <x:c r="AL225" s="6" t="s">
+        <x:v>115</x:v>
+      </x:c>
+      <x:c r="AM225" s="6" t="s">
+        <x:v>115</x:v>
+      </x:c>
+      <x:c r="AN225" s="6" t="s">
+        <x:v>115</x:v>
       </x:c>
       <x:c r="AO225" t="s">
         <x:v>1</x:v>
@@ -66003,11 +66018,11 @@
       <x:c r="AR225" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="AS225" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AT225" t="s">
-        <x:v>1</x:v>
+      <x:c r="AS225" s="6" t="s">
+        <x:v>115</x:v>
+      </x:c>
+      <x:c r="AT225" s="6" t="s">
+        <x:v>115</x:v>
       </x:c>
       <x:c r="AU225" t="s">
         <x:v>1</x:v>
@@ -66015,149 +66030,149 @@
       <x:c r="AV225" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="AW225" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AX225" t="s">
-        <x:v>1</x:v>
+      <x:c r="AW225" s="6" t="s">
+        <x:v>115</x:v>
+      </x:c>
+      <x:c r="AX225" s="6" t="s">
+        <x:v>115</x:v>
       </x:c>
       <x:c r="AY225" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="AZ225" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BA225" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BB225" t="s">
-        <x:v>1</x:v>
+      <x:c r="AZ225" s="6" t="s">
+        <x:v>115</x:v>
+      </x:c>
+      <x:c r="BA225" s="6" t="s">
+        <x:v>115</x:v>
+      </x:c>
+      <x:c r="BB225" s="6" t="s">
+        <x:v>115</x:v>
       </x:c>
       <x:c r="BC225" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="BD225" t="s">
-        <x:v>1</x:v>
+      <x:c r="BD225" s="6" t="s">
+        <x:v>115</x:v>
       </x:c>
       <x:c r="BE225" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="BF225" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BG225" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BH225" t="s">
-        <x:v>1</x:v>
+      <x:c r="BF225" s="6" t="s">
+        <x:v>115</x:v>
+      </x:c>
+      <x:c r="BG225" s="6" t="s">
+        <x:v>115</x:v>
+      </x:c>
+      <x:c r="BH225" s="6" t="s">
+        <x:v>115</x:v>
       </x:c>
       <x:c r="BI225" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="BJ225" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BK225" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BL225" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BM225" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BN225" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BO225" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BP225" t="s">
-        <x:v>1</x:v>
+      <x:c r="BJ225" s="6" t="s">
+        <x:v>115</x:v>
+      </x:c>
+      <x:c r="BK225" s="6" t="s">
+        <x:v>115</x:v>
+      </x:c>
+      <x:c r="BL225" s="6" t="s">
+        <x:v>115</x:v>
+      </x:c>
+      <x:c r="BM225" s="6" t="s">
+        <x:v>115</x:v>
+      </x:c>
+      <x:c r="BN225" s="6" t="s">
+        <x:v>115</x:v>
+      </x:c>
+      <x:c r="BO225" s="6" t="s">
+        <x:v>115</x:v>
+      </x:c>
+      <x:c r="BP225" s="6" t="s">
+        <x:v>115</x:v>
       </x:c>
       <x:c r="BQ225" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="BR225" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BS225" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BT225" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BU225" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BV225" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BW225" t="s">
-        <x:v>1</x:v>
+      <x:c r="BR225" s="6" t="s">
+        <x:v>115</x:v>
+      </x:c>
+      <x:c r="BS225" s="6" t="s">
+        <x:v>115</x:v>
+      </x:c>
+      <x:c r="BT225" s="6" t="s">
+        <x:v>115</x:v>
+      </x:c>
+      <x:c r="BU225" s="6" t="s">
+        <x:v>115</x:v>
+      </x:c>
+      <x:c r="BV225" s="6" t="s">
+        <x:v>115</x:v>
+      </x:c>
+      <x:c r="BW225" s="6" t="s">
+        <x:v>115</x:v>
       </x:c>
       <x:c r="BX225" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="BY225" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BZ225" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="CA225" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="CB225" t="s">
-        <x:v>1</x:v>
+      <x:c r="BY225" s="6" t="s">
+        <x:v>115</x:v>
+      </x:c>
+      <x:c r="BZ225" s="6" t="s">
+        <x:v>115</x:v>
+      </x:c>
+      <x:c r="CA225" s="6" t="s">
+        <x:v>115</x:v>
+      </x:c>
+      <x:c r="CB225" s="6" t="s">
+        <x:v>115</x:v>
       </x:c>
       <x:c r="CC225" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="CD225" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="CE225" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="CF225" t="s">
-        <x:v>1</x:v>
+      <x:c r="CD225" s="6" t="s">
+        <x:v>115</x:v>
+      </x:c>
+      <x:c r="CE225" s="6" t="s">
+        <x:v>115</x:v>
+      </x:c>
+      <x:c r="CF225" s="6" t="s">
+        <x:v>115</x:v>
       </x:c>
       <x:c r="CG225" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="CH225" s="6" t="s">
-        <x:v>115</x:v>
-      </x:c>
-      <x:c r="CI225" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="CJ225" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="CK225" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="CL225" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="CM225" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="CN225" t="s">
-        <x:v>1</x:v>
+      <x:c r="CH225" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="CI225" s="6" t="s">
+        <x:v>115</x:v>
+      </x:c>
+      <x:c r="CJ225" s="6" t="s">
+        <x:v>115</x:v>
+      </x:c>
+      <x:c r="CK225" s="6" t="s">
+        <x:v>115</x:v>
+      </x:c>
+      <x:c r="CL225" s="6" t="s">
+        <x:v>115</x:v>
+      </x:c>
+      <x:c r="CM225" s="6" t="s">
+        <x:v>115</x:v>
+      </x:c>
+      <x:c r="CN225" s="6" t="s">
+        <x:v>115</x:v>
       </x:c>
       <x:c r="CO225" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="CP225" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="CQ225" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="CR225" t="s">
-        <x:v>1</x:v>
+      <x:c r="CP225" s="6" t="s">
+        <x:v>115</x:v>
+      </x:c>
+      <x:c r="CQ225" s="6" t="s">
+        <x:v>115</x:v>
+      </x:c>
+      <x:c r="CR225" s="6" t="s">
+        <x:v>115</x:v>
       </x:c>
       <x:c r="CS225" t="s">
         <x:v>1</x:v>
@@ -66165,324 +66180,324 @@
       <x:c r="CT225" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="CU225" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="CV225" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="CW225" t="s">
-        <x:v>1</x:v>
+      <x:c r="CU225" s="6" t="s">
+        <x:v>115</x:v>
+      </x:c>
+      <x:c r="CV225" s="6" t="s">
+        <x:v>115</x:v>
+      </x:c>
+      <x:c r="CW225" s="6" t="s">
+        <x:v>115</x:v>
       </x:c>
     </x:row>
     <x:row r="226">
-      <x:c r="A226" s="3" t="s">
-        <x:v>466</x:v>
+      <x:c r="A226" s="4" t="s">
+        <x:v>468</x:v>
+      </x:c>
+      <x:c r="B226" s="5" t="s">
+        <x:v>469</x:v>
+      </x:c>
+      <x:c r="C226" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D226" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E226" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F226" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G226" s="6" t="s">
+        <x:v>115</x:v>
+      </x:c>
+      <x:c r="H226" s="6" t="s">
+        <x:v>115</x:v>
+      </x:c>
+      <x:c r="I226" s="6" t="s">
+        <x:v>115</x:v>
+      </x:c>
+      <x:c r="J226" s="6" t="s">
+        <x:v>115</x:v>
+      </x:c>
+      <x:c r="K226" s="6" t="s">
+        <x:v>115</x:v>
+      </x:c>
+      <x:c r="L226" s="6" t="s">
+        <x:v>115</x:v>
+      </x:c>
+      <x:c r="M226" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="N226" s="6" t="s">
+        <x:v>115</x:v>
+      </x:c>
+      <x:c r="O226" s="6" t="s">
+        <x:v>115</x:v>
+      </x:c>
+      <x:c r="P226" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="Q226" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="R226" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="S226" s="6" t="s">
+        <x:v>115</x:v>
+      </x:c>
+      <x:c r="T226" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="U226" s="6" t="s">
+        <x:v>115</x:v>
+      </x:c>
+      <x:c r="V226" s="6" t="s">
+        <x:v>115</x:v>
+      </x:c>
+      <x:c r="W226" s="6" t="s">
+        <x:v>115</x:v>
+      </x:c>
+      <x:c r="X226" s="6" t="s">
+        <x:v>115</x:v>
+      </x:c>
+      <x:c r="Y226" s="6" t="s">
+        <x:v>115</x:v>
+      </x:c>
+      <x:c r="Z226" s="6" t="s">
+        <x:v>115</x:v>
+      </x:c>
+      <x:c r="AA226" s="6" t="s">
+        <x:v>115</x:v>
+      </x:c>
+      <x:c r="AB226" s="6" t="s">
+        <x:v>115</x:v>
+      </x:c>
+      <x:c r="AC226" s="6" t="s">
+        <x:v>115</x:v>
+      </x:c>
+      <x:c r="AD226" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AE226" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AF226" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AG226" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AH226" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AI226" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AJ226" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AK226" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AL226" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AM226" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AN226" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AO226" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AP226" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AQ226" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AR226" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AS226" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AT226" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AU226" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AV226" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AW226" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AX226" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AY226" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AZ226" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BA226" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BB226" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BC226" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BD226" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BE226" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BF226" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BG226" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BH226" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BI226" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BJ226" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BK226" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BL226" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BM226" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BN226" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BO226" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BP226" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BQ226" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BR226" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BS226" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BT226" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BU226" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BV226" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BW226" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BX226" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BY226" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BZ226" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="CA226" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="CB226" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="CC226" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="CD226" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="CE226" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="CF226" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="CG226" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="CH226" s="6" t="s">
+        <x:v>115</x:v>
+      </x:c>
+      <x:c r="CI226" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="CJ226" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="CK226" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="CL226" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="CM226" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="CN226" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="CO226" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="CP226" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="CQ226" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="CR226" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="CS226" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="CT226" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="CU226" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="CV226" t="s">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="CW226" t="s">
         <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="227">
-      <x:c r="A227" s="4" t="s">
-        <x:v>467</x:v>
-      </x:c>
-      <x:c r="B227" s="5" t="s">
-        <x:v>468</x:v>
-      </x:c>
-      <x:c r="C227" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="D227" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E227" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="F227" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="G227" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="H227" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="I227" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="J227" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="K227" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="L227" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="M227" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="N227" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="O227" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="P227" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="Q227" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="R227" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="S227" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="T227" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="U227" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="V227" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="W227" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="X227" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="Y227" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="Z227" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AA227" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AB227" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AC227" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AD227" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AE227" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AF227" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AG227" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AH227" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AI227" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AJ227" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AK227" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AL227" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AM227" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AN227" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AO227" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AP227" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AQ227" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AR227" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AS227" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AT227" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AU227" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AV227" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AW227" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AX227" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AY227" s="6" t="s">
-        <x:v>115</x:v>
-      </x:c>
-      <x:c r="AZ227" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BA227" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BB227" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BC227" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BD227" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BE227" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BF227" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BG227" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BH227" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BI227" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BJ227" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BK227" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BL227" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BM227" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BN227" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BO227" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BP227" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BQ227" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BR227" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BS227" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BT227" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BU227" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BV227" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BW227" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BX227" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BY227" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BZ227" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="CA227" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="CB227" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="CC227" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="CD227" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="CE227" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="CF227" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="CG227" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="CH227" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="CI227" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="CJ227" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="CK227" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="CL227" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="CM227" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="CN227" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="CO227" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="CP227" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="CQ227" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="CR227" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="CS227" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="CT227" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="CU227" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="CV227" t="s">
-        <x:v>1</x:v>
+      <x:c r="A227" s="3" t="s">
+        <x:v>470</x:v>
       </x:c>
       <x:c r="CW227" t="s">
         <x:v>1</x:v>
@@ -66490,10 +66505,10 @@
     </x:row>
     <x:row r="228">
       <x:c r="A228" s="4" t="s">
-        <x:v>469</x:v>
+        <x:v>471</x:v>
       </x:c>
       <x:c r="B228" s="5" t="s">
-        <x:v>470</x:v>
+        <x:v>472</x:v>
       </x:c>
       <x:c r="C228" t="s">
         <x:v>1</x:v>
@@ -66639,8 +66654,8 @@
       <x:c r="AX228" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="AY228" t="s">
-        <x:v>1</x:v>
+      <x:c r="AY228" s="6" t="s">
+        <x:v>115</x:v>
       </x:c>
       <x:c r="AZ228" t="s">
         <x:v>1</x:v>
@@ -66795,10 +66810,10 @@
     </x:row>
     <x:row r="229">
       <x:c r="A229" s="4" t="s">
-        <x:v>471</x:v>
+        <x:v>473</x:v>
       </x:c>
       <x:c r="B229" s="5" t="s">
-        <x:v>472</x:v>
+        <x:v>474</x:v>
       </x:c>
       <x:c r="C229" t="s">
         <x:v>1</x:v>
@@ -66848,8 +66863,8 @@
       <x:c r="R229" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="S229" s="6" t="s">
-        <x:v>115</x:v>
+      <x:c r="S229" t="s">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="T229" t="s">
         <x:v>1</x:v>
@@ -67100,10 +67115,10 @@
     </x:row>
     <x:row r="230">
       <x:c r="A230" s="4" t="s">
-        <x:v>473</x:v>
+        <x:v>475</x:v>
       </x:c>
       <x:c r="B230" s="5" t="s">
-        <x:v>128</x:v>
+        <x:v>476</x:v>
       </x:c>
       <x:c r="C230" t="s">
         <x:v>1</x:v>
@@ -67153,8 +67168,8 @@
       <x:c r="R230" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="S230" t="s">
-        <x:v>1</x:v>
+      <x:c r="S230" s="6" t="s">
+        <x:v>115</x:v>
       </x:c>
       <x:c r="T230" t="s">
         <x:v>1</x:v>
@@ -67327,8 +67342,8 @@
       <x:c r="BX230" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="BY230" s="6" t="s">
-        <x:v>115</x:v>
+      <x:c r="BY230" t="s">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="BZ230" t="s">
         <x:v>1</x:v>
@@ -67405,16 +67420,16 @@
     </x:row>
     <x:row r="231">
       <x:c r="A231" s="4" t="s">
-        <x:v>474</x:v>
+        <x:v>477</x:v>
       </x:c>
       <x:c r="B231" s="5" t="s">
-        <x:v>475</x:v>
+        <x:v>128</x:v>
       </x:c>
       <x:c r="C231" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="D231" s="6" t="s">
-        <x:v>115</x:v>
+      <x:c r="D231" t="s">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="E231" t="s">
         <x:v>1</x:v>
@@ -67569,8 +67584,8 @@
       <x:c r="BC231" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="BD231" s="6" t="s">
-        <x:v>115</x:v>
+      <x:c r="BD231" t="s">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="BE231" t="s">
         <x:v>1</x:v>
@@ -67632,8 +67647,8 @@
       <x:c r="BX231" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="BY231" t="s">
-        <x:v>1</x:v>
+      <x:c r="BY231" s="6" t="s">
+        <x:v>115</x:v>
       </x:c>
       <x:c r="BZ231" t="s">
         <x:v>1</x:v>
@@ -67710,10 +67725,10 @@
     </x:row>
     <x:row r="232">
       <x:c r="A232" s="4" t="s">
-        <x:v>476</x:v>
+        <x:v>478</x:v>
       </x:c>
       <x:c r="B232" s="5" t="s">
-        <x:v>477</x:v>
+        <x:v>479</x:v>
       </x:c>
       <x:c r="C232" t="s">
         <x:v>1</x:v>
@@ -68015,10 +68030,10 @@
     </x:row>
     <x:row r="233">
       <x:c r="A233" s="4" t="s">
-        <x:v>478</x:v>
+        <x:v>480</x:v>
       </x:c>
       <x:c r="B233" s="5" t="s">
-        <x:v>479</x:v>
+        <x:v>481</x:v>
       </x:c>
       <x:c r="C233" t="s">
         <x:v>1</x:v>
@@ -68320,16 +68335,16 @@
     </x:row>
     <x:row r="234">
       <x:c r="A234" s="4" t="s">
-        <x:v>1</x:v>
+        <x:v>482</x:v>
       </x:c>
       <x:c r="B234" s="5" t="s">
-        <x:v>480</x:v>
+        <x:v>483</x:v>
       </x:c>
       <x:c r="C234" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="D234" t="s">
-        <x:v>1</x:v>
+      <x:c r="D234" s="6" t="s">
+        <x:v>115</x:v>
       </x:c>
       <x:c r="E234" t="s">
         <x:v>1</x:v>
@@ -68484,11 +68499,11 @@
       <x:c r="BC234" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="BD234" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BE234" s="6" t="s">
-        <x:v>115</x:v>
+      <x:c r="BD234" s="6" t="s">
+        <x:v>115</x:v>
+      </x:c>
+      <x:c r="BE234" t="s">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="BF234" t="s">
         <x:v>1</x:v>
@@ -68624,307 +68639,612 @@
       </x:c>
     </x:row>
     <x:row r="235">
-      <x:c r="A235" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="B235" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="C235" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="D235" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E235" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="F235" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="G235" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="H235" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="I235" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="J235" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="K235" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="L235" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="M235" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="N235" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="O235" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="P235" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="Q235" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="R235" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="S235" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="T235" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="U235" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="V235" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="W235" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="X235" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="Y235" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="Z235" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AA235" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AB235" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AC235" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AD235" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AE235" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AF235" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AG235" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AH235" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AI235" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AJ235" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AK235" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AL235" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AM235" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AN235" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AO235" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AP235" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AQ235" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AR235" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AS235" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AT235" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AU235" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AV235" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AW235" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AX235" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AY235" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AZ235" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BA235" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BB235" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BC235" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BD235" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BE235" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BF235" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BG235" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BH235" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BI235" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BJ235" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BK235" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BL235" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BM235" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BN235" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BO235" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BP235" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BQ235" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BR235" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BS235" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BT235" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BU235" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BV235" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BW235" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BX235" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BY235" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="BZ235" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="CA235" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="CB235" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="CC235" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="CD235" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="CE235" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="CF235" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="CG235" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="CH235" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="CI235" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="CJ235" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="CK235" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="CL235" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="CM235" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="CN235" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="CO235" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="CP235" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="CQ235" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="CR235" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="CS235" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="CT235" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="CU235" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="CV235" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="CW235" s="7" t="s">
+      <x:c r="A235" s="4" t="s">
+        <x:v>484</x:v>
+      </x:c>
+      <x:c r="B235" s="5" t="s">
+        <x:v>485</x:v>
+      </x:c>
+      <x:c r="C235" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D235" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E235" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F235" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G235" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H235" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="I235" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J235" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="K235" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="L235" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M235" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="N235" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="O235" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P235" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="Q235" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="R235" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="S235" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="T235" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="U235" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="V235" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="W235" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="X235" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="Y235" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="Z235" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AA235" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AB235" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AC235" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AD235" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AE235" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AF235" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AG235" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AH235" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AI235" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AJ235" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AK235" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AL235" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AM235" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AN235" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AO235" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AP235" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AQ235" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AR235" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AS235" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AT235" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AU235" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AV235" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AW235" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AX235" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AY235" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AZ235" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BA235" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BB235" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BC235" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BD235" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BE235" s="6" t="s">
+        <x:v>115</x:v>
+      </x:c>
+      <x:c r="BF235" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BG235" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BH235" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BI235" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BJ235" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BK235" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BL235" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BM235" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BN235" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BO235" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BP235" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BQ235" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BR235" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BS235" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BT235" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BU235" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BV235" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BW235" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BX235" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BY235" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BZ235" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="CA235" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="CB235" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="CC235" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="CD235" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="CE235" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="CF235" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="CG235" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="CH235" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="CI235" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="CJ235" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="CK235" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="CL235" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="CM235" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="CN235" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="CO235" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="CP235" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="CQ235" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="CR235" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="CS235" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="CT235" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="CU235" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="CV235" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="CW235" t="s">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="236">
+      <x:c r="A236" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B236" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C236" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D236" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E236" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F236" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G236" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H236" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="I236" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J236" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="K236" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="L236" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M236" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="N236" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="O236" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P236" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="Q236" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="R236" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="S236" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="T236" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="U236" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="V236" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="W236" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="X236" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="Y236" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="Z236" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AA236" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AB236" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AC236" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AD236" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AE236" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AF236" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AG236" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AH236" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AI236" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AJ236" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AK236" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AL236" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AM236" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AN236" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AO236" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AP236" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AQ236" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AR236" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AS236" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AT236" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AU236" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AV236" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AW236" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AX236" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AY236" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AZ236" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BA236" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BB236" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BC236" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BD236" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BE236" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BF236" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BG236" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BH236" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BI236" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BJ236" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BK236" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BL236" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BM236" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BN236" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BO236" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BP236" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BQ236" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BR236" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BS236" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BT236" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BU236" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BV236" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BW236" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BX236" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BY236" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="BZ236" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="CA236" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="CB236" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="CC236" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="CD236" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="CE236" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="CF236" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="CG236" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="CH236" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="CI236" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="CJ236" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="CK236" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="CL236" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="CM236" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="CN236" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="CO236" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="CP236" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="CQ236" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="CR236" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="CS236" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="CT236" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="CU236" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="CV236" s="7" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="CW236" s="7" t="s">
         <x:v>1</x:v>
       </x:c>
     </x:row>
@@ -68975,7 +69295,7 @@
     <x:mergeCell ref="A189:CW189"/>
     <x:mergeCell ref="A196:CW196"/>
     <x:mergeCell ref="A207:CW207"/>
-    <x:mergeCell ref="A226:CW226"/>
+    <x:mergeCell ref="A227:CW227"/>
   </x:mergeCells>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Clarify UTF-8 mode in SRELL.
</commit_message>
<xml_diff>
--- a/RegexFeatureMatrix.xlsx
+++ b/RegexFeatureMatrix.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Matrix" sheetId="1" r:id="Reaa2dd3a460e4d19"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Matrix" sheetId="1" r:id="R625b83dfd2274ee6"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -26,7 +26,7 @@
   </x:t>
   </x:si>
   <x:si>
-    <x:t>wregex
+    <x:t>std::basic_regex
   </x:t>
   </x:si>
   <x:si>
@@ -171,13 +171,13 @@
     <x:t>GCC (ECMAScript)</x:t>
   </x:si>
   <x:si>
-    <x:t>SRELL</x:t>
+    <x:t>SRELL u8</x:t>
   </x:si>
   <x:si>
-    <x:t>SRELL (“uv” flags)</x:t>
+    <x:t>SRELL u8 (“uv” flags)</x:t>
   </x:si>
   <x:si>
-    <x:t>SRELL linear (“uv” flags)</x:t>
+    <x:t>SREL3 u8 (“uv” flags)</x:t>
   </x:si>
   <x:si>
     <x:t>normal</x:t>
@@ -1633,9 +1633,9 @@
     <x:col min="11" max="11" width="5.599" customWidth="1"/>
     <x:col min="12" max="12" width="6.599" customWidth="1"/>
     <x:col min="13" max="13" width="17.48" customWidth="1"/>
-    <x:col min="14" max="14" width="7.696" customWidth="1"/>
-    <x:col min="15" max="15" width="16.787" customWidth="1"/>
-    <x:col min="16" max="16" width="21.683" customWidth="1"/>
+    <x:col min="14" max="14" width="10.196" customWidth="1"/>
+    <x:col min="15" max="15" width="19.287" customWidth="1"/>
+    <x:col min="16" max="16" width="19.287" customWidth="1"/>
     <x:col min="17" max="17" width="7.496" customWidth="1"/>
     <x:col min="18" max="18" width="6.198" customWidth="1"/>
     <x:col min="19" max="19" width="12.197" customWidth="1"/>
@@ -64095,14 +64095,14 @@
       <x:c r="M219" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="N219" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="O219" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="P219" t="s">
-        <x:v>1</x:v>
+      <x:c r="N219" s="6" t="s">
+        <x:v>115</x:v>
+      </x:c>
+      <x:c r="O219" s="6" t="s">
+        <x:v>115</x:v>
+      </x:c>
+      <x:c r="P219" s="6" t="s">
+        <x:v>115</x:v>
       </x:c>
       <x:c r="Q219" s="6" t="s">
         <x:v>115</x:v>

</xml_diff>

<commit_message>
Update RE2 engine: 2025-11-05.
</commit_message>
<xml_diff>
--- a/RegexFeatureMatrix.xlsx
+++ b/RegexFeatureMatrix.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Matrix" sheetId="1" r:id="Rbca43398504c4654"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Matrix" sheetId="1" r:id="Rf8183c257a594de9"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -31,7 +31,7 @@
   </x:si>
   <x:si>
     <x:t>RE2
- 2025-08-12 </x:t>
+ 2025-11-05 </x:t>
   </x:si>
   <x:si>
     <x:t>SubReg

</xml_diff>

<commit_message>
Update REAL engines (C++, Python, Rust): 2026.9.6.
</commit_message>
<xml_diff>
--- a/RegexFeatureMatrix.xlsx
+++ b/RegexFeatureMatrix.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Matrix" sheetId="1" r:id="Rf8183c257a594de9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Matrix" sheetId="1" r:id="Rf5cd56c236424dd5"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -135,7 +135,7 @@
   </x:si>
   <x:si>
     <x:t>REAL
- 2026.9.5 </x:t>
+ 2026.9.6 </x:t>
   </x:si>
   <x:si>
     <x:t>Regex</x:t>

</xml_diff>

<commit_message>
Update Ferroni engine: 1.5.1. Fix Feature Matrix for several engines.
</commit_message>
<xml_diff>
--- a/RegexFeatureMatrix.xlsx
+++ b/RegexFeatureMatrix.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Matrix" sheetId="1" r:id="Rf5cd56c236424dd5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Matrix" sheetId="1" r:id="Rfaf6f3804e4047a4"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -63608,8 +63608,8 @@
       <x:c r="BJ213" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="BK213" s="6" t="s">
-        <x:v>117</x:v>
+      <x:c r="BK213" t="s">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="BL213" s="6" t="s">
         <x:v>117</x:v>
@@ -67241,38 +67241,38 @@
       <x:c r="AC225" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="AD225" s="6" t="s">
-        <x:v>117</x:v>
-      </x:c>
-      <x:c r="AE225" s="6" t="s">
-        <x:v>117</x:v>
-      </x:c>
-      <x:c r="AF225" s="6" t="s">
-        <x:v>117</x:v>
-      </x:c>
-      <x:c r="AG225" s="6" t="s">
-        <x:v>117</x:v>
-      </x:c>
-      <x:c r="AH225" s="6" t="s">
-        <x:v>117</x:v>
-      </x:c>
-      <x:c r="AI225" s="6" t="s">
-        <x:v>117</x:v>
-      </x:c>
-      <x:c r="AJ225" s="6" t="s">
-        <x:v>117</x:v>
-      </x:c>
-      <x:c r="AK225" s="6" t="s">
-        <x:v>117</x:v>
-      </x:c>
-      <x:c r="AL225" s="6" t="s">
-        <x:v>117</x:v>
-      </x:c>
-      <x:c r="AM225" s="6" t="s">
-        <x:v>117</x:v>
-      </x:c>
-      <x:c r="AN225" s="6" t="s">
-        <x:v>117</x:v>
+      <x:c r="AD225" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AE225" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AF225" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AG225" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AH225" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AI225" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AJ225" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AK225" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AL225" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AM225" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AN225" t="s">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="AO225" t="s">
         <x:v>1</x:v>
@@ -67328,8 +67328,8 @@
       <x:c r="BF225" s="6" t="s">
         <x:v>117</x:v>
       </x:c>
-      <x:c r="BG225" s="6" t="s">
-        <x:v>117</x:v>
+      <x:c r="BG225" t="s">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="BH225" s="6" t="s">
         <x:v>117</x:v>
@@ -67340,8 +67340,8 @@
       <x:c r="BJ225" s="6" t="s">
         <x:v>117</x:v>
       </x:c>
-      <x:c r="BK225" s="6" t="s">
-        <x:v>117</x:v>
+      <x:c r="BK225" t="s">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="BL225" s="6" t="s">
         <x:v>117</x:v>
@@ -67361,8 +67361,8 @@
       <x:c r="BQ225" s="6" t="s">
         <x:v>117</x:v>
       </x:c>
-      <x:c r="BR225" s="6" t="s">
-        <x:v>117</x:v>
+      <x:c r="BR225" t="s">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="BS225" t="s">
         <x:v>1</x:v>
@@ -67388,8 +67388,8 @@
       <x:c r="BZ225" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="CA225" s="6" t="s">
-        <x:v>117</x:v>
+      <x:c r="CA225" t="s">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="CB225" s="6" t="s">
         <x:v>117</x:v>
@@ -67552,38 +67552,38 @@
       <x:c r="AC226" s="6" t="s">
         <x:v>117</x:v>
       </x:c>
-      <x:c r="AD226" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AE226" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AF226" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AG226" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AH226" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AI226" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AJ226" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AK226" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AL226" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AM226" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="AN226" t="s">
-        <x:v>1</x:v>
+      <x:c r="AD226" s="6" t="s">
+        <x:v>117</x:v>
+      </x:c>
+      <x:c r="AE226" s="6" t="s">
+        <x:v>117</x:v>
+      </x:c>
+      <x:c r="AF226" s="6" t="s">
+        <x:v>117</x:v>
+      </x:c>
+      <x:c r="AG226" s="6" t="s">
+        <x:v>117</x:v>
+      </x:c>
+      <x:c r="AH226" s="6" t="s">
+        <x:v>117</x:v>
+      </x:c>
+      <x:c r="AI226" s="6" t="s">
+        <x:v>117</x:v>
+      </x:c>
+      <x:c r="AJ226" s="6" t="s">
+        <x:v>117</x:v>
+      </x:c>
+      <x:c r="AK226" s="6" t="s">
+        <x:v>117</x:v>
+      </x:c>
+      <x:c r="AL226" s="6" t="s">
+        <x:v>117</x:v>
+      </x:c>
+      <x:c r="AM226" s="6" t="s">
+        <x:v>117</x:v>
+      </x:c>
+      <x:c r="AN226" s="6" t="s">
+        <x:v>117</x:v>
       </x:c>
       <x:c r="AO226" t="s">
         <x:v>1</x:v>
@@ -67651,8 +67651,8 @@
       <x:c r="BJ226" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="BK226" t="s">
-        <x:v>1</x:v>
+      <x:c r="BK226" s="6" t="s">
+        <x:v>117</x:v>
       </x:c>
       <x:c r="BL226" t="s">
         <x:v>1</x:v>

</xml_diff>

<commit_message>
Update REAL engines (C++, Python, Rust): 2026.9.8.
</commit_message>
<xml_diff>
--- a/RegexFeatureMatrix.xlsx
+++ b/RegexFeatureMatrix.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Matrix" sheetId="1" r:id="R782afb7a0f6e4801"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Matrix" sheetId="1" r:id="Rde0100cf85494805"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -135,7 +135,7 @@
   </x:si>
   <x:si>
     <x:t>REAL
- 2026.9.7 </x:t>
+ 2026.9.8 </x:t>
   </x:si>
   <x:si>
     <x:t>Regex</x:t>

</xml_diff>

<commit_message>
Update Rust 1.99.0, 'ferroni' 1.10.0, REAL 2026.10.5.
</commit_message>
<xml_diff>
--- a/RegexFeatureMatrix.xlsx
+++ b/RegexFeatureMatrix.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Matrix" sheetId="1" r:id="Rbac8d79028df4a51"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Matrix" sheetId="1" r:id="Rdf6eaf36f8cb4f2e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -71,7 +71,7 @@
   </x:si>
   <x:si>
     <x:t>Rust
- 1.98.1 </x:t>
+ 1.99.0 </x:t>
   </x:si>
   <x:si>
     <x:t>Java
@@ -135,7 +135,7 @@
   </x:si>
   <x:si>
     <x:t>REAL
- 2026.10.4 </x:t>
+ 2026.10.5 </x:t>
   </x:si>
   <x:si>
     <x:t>Regex</x:t>

</xml_diff>

<commit_message>
Update 'REAL' 2026-10-14 and add new limits.
</commit_message>
<xml_diff>
--- a/RegexFeatureMatrix.xlsx
+++ b/RegexFeatureMatrix.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Matrix" sheetId="1" r:id="R93a273e3b7224560"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Matrix" sheetId="1" r:id="Rb286cdb9528d4ddb"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -135,7 +135,7 @@
   </x:si>
   <x:si>
     <x:t>REAL
- 2026.10.11 </x:t>
+ 2026.10.14 </x:t>
   </x:si>
   <x:si>
     <x:t>Regex</x:t>

</xml_diff>

<commit_message>
Add “possessive” option to 'z-regex'.
</commit_message>
<xml_diff>
--- a/RegexFeatureMatrix.xlsx
+++ b/RegexFeatureMatrix.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Matrix" sheetId="1" r:id="R917c174c83c44405"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Matrix" sheetId="1" r:id="Rf1f7add8106e4c69"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -6235,6 +6235,9 @@
       <x:c r="CN34" s="6" t="s">
         <x:v>124</x:v>
       </x:c>
+      <x:c r="CR34" s="6" t="s">
+        <x:v>124</x:v>
+      </x:c>
       <x:c r="CU34" s="6" t="s">
         <x:v>124</x:v>
       </x:c>

</xml_diff>

<commit_message>
Update Rust 1.99.1, 'fancy-regex' 0.20.0, 'real-regex' 2026.10.18, 'ferroni' 2.5.2.
</commit_message>
<xml_diff>
--- a/RegexFeatureMatrix.xlsx
+++ b/RegexFeatureMatrix.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Matrix" sheetId="1" r:id="R3e798e5ecd124e15"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Matrix" sheetId="1" r:id="R65890fb1fe624ac5"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -71,7 +71,7 @@
   </x:si>
   <x:si>
     <x:t>Rust
- 1.99.0 </x:t>
+ 1.99.1 </x:t>
   </x:si>
   <x:si>
     <x:t>Java

</xml_diff>

<commit_message>
New Feature Matrix indicator: “Support sticky mode”.
</commit_message>
<xml_diff>
--- a/RegexFeatureMatrix.xlsx
+++ b/RegexFeatureMatrix.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Matrix" sheetId="1" r:id="R2854feb03d5b472a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Matrix" sheetId="1" r:id="R65a0c0ea90fc40ff"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1375,6 +1375,12 @@
   </x:si>
   <x:si>
     <x:t>Miscellaneous</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Sticky</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Support Sticky mode by “\G”, “(?y)” or an option</x:t>
   </x:si>
   <x:si>
     <x:t>Captures</x:t>
@@ -23160,21 +23166,84 @@
       <x:c r="C208" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
+      <x:c r="F208" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="G208" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="J208" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
       <x:c r="K208" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
+      <x:c r="L208" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="M208" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="N208" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="O208" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="P208" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="Q208" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="R208" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="S208" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="T208" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="U208" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="Y208" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
       <x:c r="Z208" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
       <x:c r="AA208" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
+      <x:c r="AB208" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="AC208" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="AD208" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="AE208" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="AF208" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="AG208" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
       <x:c r="AH208" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
       <x:c r="AI208" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
+      <x:c r="AN208" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
       <x:c r="AO208" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
@@ -23190,13 +23259,73 @@
       <x:c r="AS208" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
+      <x:c r="AT208" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="AU208" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="AV208" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="AW208" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="AX208" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="AZ208" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="BD208" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="BE208" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="BH208" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="BM208" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="BQ208" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
       <x:c r="BR208" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
+      <x:c r="BT208" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="BX208" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
       <x:c r="BZ208" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
       <x:c r="CA208" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="CD208" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="CN208" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="CO208" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="CW208" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="CZ208" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="DC208" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="DF208" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
     </x:row>
@@ -23210,105 +23339,21 @@
       <x:c r="C209" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
-      <x:c r="E209" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="G209" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="I209" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="J209" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
       <x:c r="K209" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
-      <x:c r="L209" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="M209" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="N209" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="O209" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="P209" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="Q209" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="R209" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="S209" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="T209" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="U209" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="V209" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="W209" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="Y209" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
       <x:c r="Z209" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
       <x:c r="AA209" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
-      <x:c r="AB209" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="AC209" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="AD209" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="AE209" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="AF209" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="AG209" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
       <x:c r="AH209" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
       <x:c r="AI209" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
-      <x:c r="AJ209" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="AK209" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="AL209" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="AM209" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="AN209" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
       <x:c r="AO209" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
@@ -23324,151 +23369,13 @@
       <x:c r="AS209" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
-      <x:c r="AT209" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="AU209" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="AV209" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="AW209" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="AX209" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="AY209" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="AZ209" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="BD209" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="BE209" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="BF209" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="BG209" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="BH209" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="BI209" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="BL209" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="BM209" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="BN209" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="BO209" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="BQ209" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
       <x:c r="BR209" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
-      <x:c r="BT209" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="BU209" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="BV209" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="BW209" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="BX209" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="BY209" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
       <x:c r="BZ209" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
       <x:c r="CA209" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="CB209" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="CD209" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="CH209" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="CI209" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="CM209" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="CO209" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="CP209" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="CQ209" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="CU209" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="CV209" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="CW209" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="CX209" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="CY209" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="CZ209" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="DA209" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="DB209" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="DC209" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="DD209" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="DE209" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="DF209" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="DH209" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="DI209" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
     </x:row>
@@ -23479,9 +23386,60 @@
       <x:c r="B210" s="5" t="s">
         <x:v>451</x:v>
       </x:c>
+      <x:c r="C210" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="E210" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="G210" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="I210" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="J210" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
       <x:c r="K210" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
+      <x:c r="L210" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="M210" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="N210" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="O210" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="P210" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="Q210" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="R210" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="S210" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="T210" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="U210" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="V210" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="W210" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
       <x:c r="Y210" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
@@ -23491,49 +23449,205 @@
       <x:c r="AA210" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
+      <x:c r="AB210" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="AC210" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="AD210" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="AE210" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="AF210" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="AG210" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="AH210" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
       <x:c r="AI210" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
+      <x:c r="AJ210" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="AK210" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="AL210" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="AM210" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="AN210" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="AO210" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
       <x:c r="AP210" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
       <x:c r="AQ210" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
+      <x:c r="AR210" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
       <x:c r="AS210" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
-      <x:c r="BC210" s="6" t="s">
+      <x:c r="AT210" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="AU210" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="AV210" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="AW210" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="AX210" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="AY210" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="AZ210" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
       <x:c r="BD210" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
+      <x:c r="BE210" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="BF210" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="BG210" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
       <x:c r="BH210" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
+      <x:c r="BI210" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="BL210" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="BM210" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="BN210" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="BO210" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
       <x:c r="BQ210" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
       <x:c r="BR210" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
+      <x:c r="BT210" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="BU210" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="BV210" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="BW210" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="BX210" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="BY210" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
       <x:c r="BZ210" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
       <x:c r="CA210" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
+      <x:c r="CB210" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
       <x:c r="CD210" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
-      <x:c r="CN210" s="6" t="s">
+      <x:c r="CH210" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="CI210" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="CM210" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
       <x:c r="CO210" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
+      <x:c r="CP210" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="CQ210" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="CU210" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="CV210" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="CW210" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="CX210" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="CY210" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="CZ210" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="DA210" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="DB210" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="DC210" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="DD210" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="DE210" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
       <x:c r="DF210" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="DH210" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="DI210" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
     </x:row>
@@ -23544,13 +23658,61 @@
       <x:c r="B211" s="5" t="s">
         <x:v>453</x:v>
       </x:c>
+      <x:c r="K211" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
       <x:c r="Y211" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
+      <x:c r="Z211" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="AA211" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="AI211" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="AP211" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="AQ211" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="AS211" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="BC211" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="BD211" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="BH211" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="BQ211" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="BR211" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="BZ211" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="CA211" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
       <x:c r="CD211" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
+      <x:c r="CN211" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
       <x:c r="CO211" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="DF211" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
     </x:row>
@@ -23564,16 +23726,10 @@
       <x:c r="Y212" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
-      <x:c r="AI212" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="AP212" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="AQ212" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="AS212" s="6" t="s">
+      <x:c r="CD212" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="CO212" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
     </x:row>
@@ -23584,76 +23740,19 @@
       <x:c r="B213" s="5" t="s">
         <x:v>457</x:v>
       </x:c>
-      <x:c r="K213" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="V213" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
       <x:c r="Y213" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
-      <x:c r="AY213" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="BB213" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="BC213" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="BD213" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="BM213" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="BR213" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="BT213" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="BU213" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="BV213" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="BZ213" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="CA213" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="CD213" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="CI213" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="CN213" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="CO213" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="CQ213" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="CS213" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="CV213" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="CX213" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="DB213" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="DF213" s="6" t="s">
+      <x:c r="AI213" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="AP213" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="AQ213" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="AS213" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
     </x:row>
@@ -23664,88 +23763,76 @@
       <x:c r="B214" s="5" t="s">
         <x:v>459</x:v>
       </x:c>
-      <x:c r="G214" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="J214" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="L214" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="R214" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="S214" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="T214" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="U214" s="6" t="s">
+      <x:c r="K214" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="V214" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
       <x:c r="Y214" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
-      <x:c r="AT214" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="AU214" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="AV214" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="AW214" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="AX214" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="AZ214" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="BI214" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="BK214" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="BW214" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="CF214" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="CJ214" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="CK214" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="CL214" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="CR214" s="6" t="s">
+      <x:c r="AY214" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="BB214" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="BC214" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="BD214" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="BM214" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="BR214" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="BT214" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="BU214" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="BV214" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="BZ214" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="CA214" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="CD214" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="CI214" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="CN214" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="CO214" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="CQ214" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
       <x:c r="CS214" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
-      <x:c r="CW214" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="DA214" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="DD214" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="DE214" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="DG214" s="6" t="s">
+      <x:c r="CV214" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="CX214" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="DB214" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="DF214" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
     </x:row>
@@ -23804,9 +23891,6 @@
       <x:c r="BK215" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
-      <x:c r="BO215" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
       <x:c r="BW215" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
@@ -23820,9 +23904,6 @@
         <x:v>129</x:v>
       </x:c>
       <x:c r="CL215" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="CP215" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
       <x:c r="CR215" s="6" t="s">
@@ -23854,51 +23935,15 @@
       <x:c r="B216" s="5" t="s">
         <x:v>463</x:v>
       </x:c>
-      <x:c r="C216" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="D216" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="E216" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="F216" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
       <x:c r="G216" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
-      <x:c r="H216" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="I216" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
       <x:c r="J216" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
-      <x:c r="K216" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
       <x:c r="L216" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
-      <x:c r="M216" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="N216" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="O216" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="P216" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="Q216" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
       <x:c r="R216" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
@@ -23911,75 +23956,9 @@
       <x:c r="U216" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
-      <x:c r="V216" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="W216" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
       <x:c r="Y216" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
-      <x:c r="Z216" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="AA216" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="AB216" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="AC216" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="AD216" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="AE216" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="AF216" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="AG216" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="AH216" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="AI216" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="AJ216" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="AK216" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="AL216" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="AM216" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="AN216" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="AO216" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="AP216" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="AQ216" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="AR216" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="AS216" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
       <x:c r="AT216" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
@@ -23995,169 +23974,55 @@
       <x:c r="AX216" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
-      <x:c r="AY216" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
       <x:c r="AZ216" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
-      <x:c r="BA216" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="BB216" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="BC216" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="BD216" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="BE216" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="BF216" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="BG216" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="BH216" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
       <x:c r="BI216" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
-      <x:c r="BJ216" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
       <x:c r="BK216" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
-      <x:c r="BL216" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="BM216" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="BN216" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
       <x:c r="BO216" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
-      <x:c r="BP216" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="BQ216" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="BR216" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="BS216" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="BT216" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="BU216" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="BV216" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
       <x:c r="BW216" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
-      <x:c r="BX216" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="BY216" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="BZ216" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="CA216" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="CB216" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="CC216" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="CD216" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="CE216" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="CH216" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="CI216" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="CN216" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="CO216" s="6" t="s">
+      <x:c r="CF216" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="CJ216" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="CK216" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="CL216" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
       <x:c r="CP216" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
-      <x:c r="CQ216" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
       <x:c r="CR216" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
-      <x:c r="CU216" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="CV216" s="6" t="s">
+      <x:c r="CS216" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
       <x:c r="CW216" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
-      <x:c r="CX216" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="CY216" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="CZ216" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
       <x:c r="DA216" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
-      <x:c r="DB216" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="DC216" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
       <x:c r="DD216" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
       <x:c r="DE216" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
-      <x:c r="DF216" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
       <x:c r="DG216" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="DH216" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="DI216" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
     </x:row>
@@ -24180,21 +24045,57 @@
       <x:c r="F217" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
+      <x:c r="G217" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
       <x:c r="H217" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
       <x:c r="I217" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
+      <x:c r="J217" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
       <x:c r="K217" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
       <x:c r="L217" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
+      <x:c r="M217" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="N217" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="O217" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="P217" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="Q217" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
       <x:c r="R217" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
+      <x:c r="S217" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="T217" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="U217" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="V217" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="W217" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
       <x:c r="Y217" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
@@ -24213,12 +24114,30 @@
       <x:c r="AD217" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
+      <x:c r="AE217" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="AF217" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="AG217" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
       <x:c r="AH217" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
       <x:c r="AI217" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
+      <x:c r="AJ217" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="AK217" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="AL217" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
       <x:c r="AM217" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
@@ -24240,6 +24159,33 @@
       <x:c r="AS217" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
+      <x:c r="AT217" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="AU217" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="AV217" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="AW217" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="AX217" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="AY217" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="AZ217" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="BA217" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="BB217" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
       <x:c r="BC217" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
@@ -24252,12 +24198,21 @@
       <x:c r="BF217" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
+      <x:c r="BG217" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
       <x:c r="BH217" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
+      <x:c r="BI217" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
       <x:c r="BJ217" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
+      <x:c r="BK217" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
       <x:c r="BL217" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
@@ -24267,6 +24222,12 @@
       <x:c r="BN217" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
+      <x:c r="BO217" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="BP217" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
       <x:c r="BQ217" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
@@ -24279,9 +24240,15 @@
       <x:c r="BT217" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
+      <x:c r="BU217" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
       <x:c r="BV217" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
+      <x:c r="BW217" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
       <x:c r="BX217" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
@@ -24303,16 +24270,70 @@
       <x:c r="CD217" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
+      <x:c r="CE217" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="CH217" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="CI217" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="CN217" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
       <x:c r="CO217" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
+      <x:c r="CP217" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="CQ217" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="CR217" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
       <x:c r="CU217" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
+      <x:c r="CV217" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="CW217" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="CX217" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="CY217" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
       <x:c r="CZ217" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
+      <x:c r="DA217" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="DB217" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="DC217" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="DD217" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="DE217" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
       <x:c r="DF217" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="DG217" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="DH217" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
       <x:c r="DI217" s="6" t="s">
@@ -24338,57 +24359,21 @@
       <x:c r="F218" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
-      <x:c r="G218" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
       <x:c r="H218" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
       <x:c r="I218" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
-      <x:c r="J218" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
       <x:c r="K218" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
       <x:c r="L218" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
-      <x:c r="M218" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="N218" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="O218" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="P218" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="Q218" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
       <x:c r="R218" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
-      <x:c r="S218" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="T218" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="U218" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="V218" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="W218" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
       <x:c r="Y218" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
@@ -24407,30 +24392,12 @@
       <x:c r="AD218" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
-      <x:c r="AE218" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="AF218" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="AG218" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
       <x:c r="AH218" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
       <x:c r="AI218" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
-      <x:c r="AJ218" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="AK218" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="AL218" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
       <x:c r="AM218" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
@@ -24452,33 +24419,6 @@
       <x:c r="AS218" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
-      <x:c r="AT218" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="AU218" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="AV218" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="AW218" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="AX218" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="AY218" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="AZ218" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="BA218" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="BB218" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
       <x:c r="BC218" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
@@ -24491,21 +24431,12 @@
       <x:c r="BF218" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
-      <x:c r="BG218" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
       <x:c r="BH218" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
-      <x:c r="BI218" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
       <x:c r="BJ218" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
-      <x:c r="BK218" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
       <x:c r="BL218" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
@@ -24515,12 +24446,6 @@
       <x:c r="BN218" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
-      <x:c r="BO218" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="BP218" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
       <x:c r="BQ218" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
@@ -24533,15 +24458,9 @@
       <x:c r="BT218" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
-      <x:c r="BU218" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
       <x:c r="BV218" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
-      <x:c r="BW218" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
       <x:c r="BX218" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
@@ -24563,70 +24482,16 @@
       <x:c r="CD218" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
-      <x:c r="CE218" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="CH218" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="CI218" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="CN218" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
       <x:c r="CO218" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
-      <x:c r="CP218" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="CQ218" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="CR218" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
       <x:c r="CU218" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
-      <x:c r="CV218" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="CW218" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="CX218" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="CY218" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
       <x:c r="CZ218" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
-      <x:c r="DA218" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="DB218" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="DC218" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="DD218" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="DE218" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
       <x:c r="DF218" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="DG218" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="DH218" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
       <x:c r="DI218" s="6" t="s">
@@ -24640,9 +24505,18 @@
       <x:c r="B219" s="5" t="s">
         <x:v>469</x:v>
       </x:c>
+      <x:c r="C219" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="D219" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
       <x:c r="E219" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
+      <x:c r="F219" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
       <x:c r="G219" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
@@ -24658,6 +24532,27 @@
       <x:c r="K219" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
+      <x:c r="L219" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="M219" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="N219" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="O219" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="P219" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="Q219" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="R219" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
       <x:c r="S219" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
@@ -24676,6 +24571,33 @@
       <x:c r="Y219" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
+      <x:c r="Z219" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="AA219" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="AB219" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="AC219" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="AD219" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="AE219" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="AF219" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="AG219" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="AH219" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
       <x:c r="AI219" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
@@ -24709,6 +24631,9 @@
       <x:c r="AS219" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
+      <x:c r="AT219" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
       <x:c r="AU219" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
@@ -24727,6 +24652,12 @@
       <x:c r="AZ219" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
+      <x:c r="BA219" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="BB219" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
       <x:c r="BC219" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
@@ -24787,6 +24718,9 @@
       <x:c r="BV219" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
+      <x:c r="BW219" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
       <x:c r="BX219" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
@@ -24811,12 +24745,27 @@
       <x:c r="CE219" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
+      <x:c r="CH219" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="CI219" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
       <x:c r="CN219" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
       <x:c r="CO219" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
+      <x:c r="CP219" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="CQ219" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="CR219" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
       <x:c r="CU219" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
@@ -24842,6 +24791,9 @@
         <x:v>129</x:v>
       </x:c>
       <x:c r="DC219" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="DD219" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
       <x:c r="DE219" s="6" t="s">
@@ -24867,21 +24819,15 @@
       <x:c r="B220" s="5" t="s">
         <x:v>471</x:v>
       </x:c>
-      <x:c r="C220" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="D220" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
       <x:c r="E220" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
-      <x:c r="F220" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
       <x:c r="G220" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
+      <x:c r="H220" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
       <x:c r="I220" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
@@ -24909,33 +24855,6 @@
       <x:c r="Y220" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
-      <x:c r="Z220" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="AA220" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="AB220" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="AC220" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="AD220" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="AE220" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="AF220" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="AG220" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="AH220" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
       <x:c r="AI220" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
@@ -24969,9 +24888,6 @@
       <x:c r="AS220" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
-      <x:c r="AT220" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
       <x:c r="AU220" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
@@ -24990,12 +24906,6 @@
       <x:c r="AZ220" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
-      <x:c r="BA220" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="BB220" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
       <x:c r="BC220" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
@@ -25008,6 +24918,9 @@
       <x:c r="BF220" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
+      <x:c r="BG220" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
       <x:c r="BH220" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
@@ -25017,6 +24930,9 @@
       <x:c r="BJ220" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
+      <x:c r="BK220" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
       <x:c r="BL220" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
@@ -25029,6 +24945,9 @@
       <x:c r="BO220" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
+      <x:c r="BP220" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
       <x:c r="BQ220" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
@@ -25047,9 +24966,6 @@
       <x:c r="BV220" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
-      <x:c r="BW220" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
       <x:c r="BX220" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
@@ -25071,15 +24987,15 @@
       <x:c r="CD220" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
+      <x:c r="CE220" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
       <x:c r="CN220" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
       <x:c r="CO220" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
-      <x:c r="CR220" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
       <x:c r="CU220" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
@@ -25092,6 +25008,9 @@
       <x:c r="CX220" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
+      <x:c r="CY220" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
       <x:c r="CZ220" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
@@ -25104,13 +25023,16 @@
       <x:c r="DC220" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
-      <x:c r="DD220" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
       <x:c r="DE220" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
       <x:c r="DF220" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="DG220" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="DH220" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
       <x:c r="DI220" s="6" t="s">
@@ -25124,7 +25046,253 @@
       <x:c r="B221" s="5" t="s">
         <x:v>473</x:v>
       </x:c>
+      <x:c r="C221" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="D221" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="E221" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="F221" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="G221" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="I221" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="J221" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="K221" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="S221" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="T221" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="U221" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="V221" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="W221" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="Y221" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="Z221" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="AA221" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="AB221" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="AC221" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="AD221" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="AE221" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="AF221" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="AG221" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="AH221" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="AI221" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="AJ221" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="AK221" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="AL221" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="AM221" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="AN221" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="AO221" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="AP221" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="AQ221" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="AR221" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="AS221" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="AT221" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="AU221" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="AV221" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="AW221" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="AX221" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="AY221" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="AZ221" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="BA221" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="BB221" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="BC221" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="BD221" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="BE221" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="BF221" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="BH221" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="BI221" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="BJ221" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="BL221" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="BM221" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="BN221" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="BO221" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="BQ221" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="BR221" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="BS221" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
       <x:c r="BT221" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="BU221" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="BV221" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="BW221" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="BX221" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="BY221" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="BZ221" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="CA221" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="CB221" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="CC221" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="CD221" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="CN221" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="CO221" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="CR221" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="CU221" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="CV221" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="CW221" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="CX221" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="CZ221" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="DA221" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="DB221" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="DC221" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="DD221" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="DE221" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="DF221" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="DI221" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
     </x:row>
@@ -25135,202 +25303,7 @@
       <x:c r="B222" s="5" t="s">
         <x:v>475</x:v>
       </x:c>
-      <x:c r="E222" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="G222" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="I222" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="J222" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="K222" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="S222" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="T222" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="U222" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="V222" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="W222" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="Y222" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="AI222" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="AJ222" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="AK222" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="AL222" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="AM222" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="AN222" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="AO222" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="AP222" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="AQ222" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="AR222" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="AS222" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="AT222" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="AU222" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="AV222" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="AW222" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="AX222" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="AY222" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="AZ222" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="BB222" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="BC222" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="BD222" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="BE222" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="BF222" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="BH222" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="BI222" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="BJ222" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="BL222" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="BM222" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="BN222" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="BQ222" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="BS222" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
       <x:c r="BT222" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="BU222" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="BV222" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="BX222" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="BY222" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="BZ222" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="CA222" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="CB222" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="CC222" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="CD222" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="CN222" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="CO222" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="CR222" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="CU222" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="CV222" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="CW222" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="CX222" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="CZ222" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="DB222" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="DC222" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="DD222" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="DE222" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="DF222" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="DI222" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
     </x:row>
@@ -25341,9 +25314,39 @@
       <x:c r="B223" s="5" t="s">
         <x:v>477</x:v>
       </x:c>
+      <x:c r="E223" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="G223" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="I223" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="J223" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
       <x:c r="K223" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
+      <x:c r="S223" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="T223" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="U223" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="V223" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="W223" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="Y223" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
       <x:c r="AI223" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
@@ -25377,28 +25380,136 @@
       <x:c r="AS223" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
+      <x:c r="AT223" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="AU223" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="AV223" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="AW223" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="AX223" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="AY223" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="AZ223" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="BB223" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="BC223" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="BD223" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
       <x:c r="BE223" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
+      <x:c r="BF223" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="BH223" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="BI223" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="BJ223" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="BL223" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="BM223" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="BN223" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
       <x:c r="BQ223" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
+      <x:c r="BS223" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="BT223" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="BU223" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="BV223" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
       <x:c r="BX223" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
+      <x:c r="BY223" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
       <x:c r="BZ223" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
       <x:c r="CA223" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
+      <x:c r="CB223" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="CC223" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
       <x:c r="CD223" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
+      <x:c r="CN223" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="CO223" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="CR223" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
       <x:c r="CU223" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
+      <x:c r="CV223" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="CW223" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="CX223" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="CZ223" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="DB223" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="DC223" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="DD223" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="DE223" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
       <x:c r="DF223" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="DI223" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
     </x:row>
@@ -25409,182 +25520,50 @@
       <x:c r="B224" s="5" t="s">
         <x:v>479</x:v>
       </x:c>
-      <x:c r="D224" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="E224" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="G224" s="7" t="s">
-        <x:v>480</x:v>
-      </x:c>
-      <x:c r="H224" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="I224" s="7" t="s">
-        <x:v>480</x:v>
-      </x:c>
-      <x:c r="J224" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
       <x:c r="K224" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
-      <x:c r="L224" s="7" t="s">
-        <x:v>480</x:v>
-      </x:c>
-      <x:c r="M224" s="7" t="s">
-        <x:v>480</x:v>
-      </x:c>
-      <x:c r="N224" s="7" t="s">
-        <x:v>480</x:v>
-      </x:c>
-      <x:c r="O224" s="7" t="s">
-        <x:v>480</x:v>
-      </x:c>
-      <x:c r="P224" s="7" t="s">
-        <x:v>480</x:v>
-      </x:c>
-      <x:c r="Q224" s="7" t="s">
-        <x:v>480</x:v>
-      </x:c>
-      <x:c r="S224" s="7" t="s">
-        <x:v>480</x:v>
-      </x:c>
-      <x:c r="T224" s="7" t="s">
-        <x:v>480</x:v>
-      </x:c>
-      <x:c r="U224" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="V224" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="W224" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="X224" s="7" t="s">
-        <x:v>480</x:v>
-      </x:c>
-      <x:c r="Y224" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="Z224" s="7" t="s">
-        <x:v>480</x:v>
-      </x:c>
-      <x:c r="AA224" s="7" t="s">
-        <x:v>480</x:v>
-      </x:c>
-      <x:c r="AB224" s="7" t="s">
-        <x:v>480</x:v>
-      </x:c>
-      <x:c r="AC224" s="7" t="s">
-        <x:v>480</x:v>
-      </x:c>
-      <x:c r="AD224" s="7" t="s">
-        <x:v>480</x:v>
-      </x:c>
-      <x:c r="AE224" s="7" t="s">
-        <x:v>480</x:v>
-      </x:c>
-      <x:c r="AF224" s="7" t="s">
-        <x:v>480</x:v>
-      </x:c>
-      <x:c r="AG224" s="7" t="s">
-        <x:v>480</x:v>
-      </x:c>
-      <x:c r="AH224" s="7" t="s">
-        <x:v>480</x:v>
-      </x:c>
-      <x:c r="AI224" s="7" t="s">
-        <x:v>480</x:v>
+      <x:c r="AI224" s="6" t="s">
+        <x:v>129</x:v>
       </x:c>
       <x:c r="AJ224" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
-      <x:c r="AK224" s="7" t="s">
-        <x:v>480</x:v>
-      </x:c>
-      <x:c r="AL224" s="7" t="s">
-        <x:v>480</x:v>
+      <x:c r="AK224" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="AL224" s="6" t="s">
+        <x:v>129</x:v>
       </x:c>
       <x:c r="AM224" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
-      <x:c r="AN224" s="7" t="s">
-        <x:v>480</x:v>
-      </x:c>
-      <x:c r="AO224" s="7" t="s">
-        <x:v>480</x:v>
-      </x:c>
-      <x:c r="AP224" s="7" t="s">
-        <x:v>480</x:v>
-      </x:c>
-      <x:c r="AQ224" s="7" t="s">
-        <x:v>480</x:v>
-      </x:c>
-      <x:c r="AR224" s="7" t="s">
-        <x:v>480</x:v>
-      </x:c>
-      <x:c r="AS224" s="7" t="s">
-        <x:v>480</x:v>
-      </x:c>
-      <x:c r="AX224" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="AY224" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="BB224" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="BC224" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="BD224" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="BF224" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="BG224" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="BH224" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="BJ224" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="BL224" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="BN224" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="BP224" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="BQ224" s="7" t="s">
-        <x:v>480</x:v>
-      </x:c>
-      <x:c r="BR224" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="BS224" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="BT224" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="BU224" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="BV224" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="BW224" s="7" t="s">
-        <x:v>480</x:v>
+      <x:c r="AN224" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="AO224" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="AP224" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="AQ224" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="AR224" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="AS224" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="BE224" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="BQ224" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="BX224" s="6" t="s">
+        <x:v>129</x:v>
       </x:c>
       <x:c r="BZ224" s="6" t="s">
         <x:v>129</x:v>
@@ -25592,114 +25571,288 @@
       <x:c r="CA224" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
-      <x:c r="CB224" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="CC224" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
       <x:c r="CD224" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
-      <x:c r="CE224" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="CH224" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="CI224" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="CK224" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="CL224" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="CN224" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="CO224" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="CP224" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="CR224" s="7" t="s">
-        <x:v>480</x:v>
-      </x:c>
-      <x:c r="CS224" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="CT224" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
       <x:c r="CU224" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
-      <x:c r="CV224" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="CW224" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="CX224" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="CY224" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="DA224" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="DB224" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="DC224" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
       <x:c r="DF224" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="DH224" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="DI224" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
     </x:row>
     <x:row r="225">
-      <x:c r="A225" s="3" t="s">
+      <x:c r="A225" s="4" t="s">
+        <x:v>480</x:v>
+      </x:c>
+      <x:c r="B225" s="5" t="s">
         <x:v>481</x:v>
       </x:c>
-      <x:c r="DI225" t="s">
-        <x:v>1</x:v>
+      <x:c r="D225" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="E225" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="G225" s="7" t="s">
+        <x:v>482</x:v>
+      </x:c>
+      <x:c r="H225" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="I225" s="7" t="s">
+        <x:v>482</x:v>
+      </x:c>
+      <x:c r="J225" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="K225" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="L225" s="7" t="s">
+        <x:v>482</x:v>
+      </x:c>
+      <x:c r="M225" s="7" t="s">
+        <x:v>482</x:v>
+      </x:c>
+      <x:c r="N225" s="7" t="s">
+        <x:v>482</x:v>
+      </x:c>
+      <x:c r="O225" s="7" t="s">
+        <x:v>482</x:v>
+      </x:c>
+      <x:c r="P225" s="7" t="s">
+        <x:v>482</x:v>
+      </x:c>
+      <x:c r="Q225" s="7" t="s">
+        <x:v>482</x:v>
+      </x:c>
+      <x:c r="S225" s="7" t="s">
+        <x:v>482</x:v>
+      </x:c>
+      <x:c r="T225" s="7" t="s">
+        <x:v>482</x:v>
+      </x:c>
+      <x:c r="U225" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="V225" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="W225" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="X225" s="7" t="s">
+        <x:v>482</x:v>
+      </x:c>
+      <x:c r="Y225" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="Z225" s="7" t="s">
+        <x:v>482</x:v>
+      </x:c>
+      <x:c r="AA225" s="7" t="s">
+        <x:v>482</x:v>
+      </x:c>
+      <x:c r="AB225" s="7" t="s">
+        <x:v>482</x:v>
+      </x:c>
+      <x:c r="AC225" s="7" t="s">
+        <x:v>482</x:v>
+      </x:c>
+      <x:c r="AD225" s="7" t="s">
+        <x:v>482</x:v>
+      </x:c>
+      <x:c r="AE225" s="7" t="s">
+        <x:v>482</x:v>
+      </x:c>
+      <x:c r="AF225" s="7" t="s">
+        <x:v>482</x:v>
+      </x:c>
+      <x:c r="AG225" s="7" t="s">
+        <x:v>482</x:v>
+      </x:c>
+      <x:c r="AH225" s="7" t="s">
+        <x:v>482</x:v>
+      </x:c>
+      <x:c r="AI225" s="7" t="s">
+        <x:v>482</x:v>
+      </x:c>
+      <x:c r="AJ225" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="AK225" s="7" t="s">
+        <x:v>482</x:v>
+      </x:c>
+      <x:c r="AL225" s="7" t="s">
+        <x:v>482</x:v>
+      </x:c>
+      <x:c r="AM225" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="AN225" s="7" t="s">
+        <x:v>482</x:v>
+      </x:c>
+      <x:c r="AO225" s="7" t="s">
+        <x:v>482</x:v>
+      </x:c>
+      <x:c r="AP225" s="7" t="s">
+        <x:v>482</x:v>
+      </x:c>
+      <x:c r="AQ225" s="7" t="s">
+        <x:v>482</x:v>
+      </x:c>
+      <x:c r="AR225" s="7" t="s">
+        <x:v>482</x:v>
+      </x:c>
+      <x:c r="AS225" s="7" t="s">
+        <x:v>482</x:v>
+      </x:c>
+      <x:c r="AX225" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="AY225" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="BB225" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="BC225" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="BD225" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="BF225" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="BG225" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="BH225" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="BJ225" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="BL225" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="BN225" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="BP225" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="BQ225" s="7" t="s">
+        <x:v>482</x:v>
+      </x:c>
+      <x:c r="BR225" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="BS225" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="BT225" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="BU225" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="BV225" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="BW225" s="7" t="s">
+        <x:v>482</x:v>
+      </x:c>
+      <x:c r="BZ225" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="CA225" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="CB225" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="CC225" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="CD225" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="CE225" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="CH225" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="CI225" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="CK225" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="CL225" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="CN225" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="CO225" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="CP225" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="CR225" s="7" t="s">
+        <x:v>482</x:v>
+      </x:c>
+      <x:c r="CS225" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="CT225" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="CU225" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="CV225" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="CW225" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="CX225" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="CY225" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="DA225" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="DB225" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="DC225" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="DF225" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="DH225" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="DI225" s="6" t="s">
+        <x:v>129</x:v>
       </x:c>
     </x:row>
     <x:row r="226">
-      <x:c r="A226" s="4" t="s">
-        <x:v>482</x:v>
-      </x:c>
-      <x:c r="B226" s="5" t="s">
+      <x:c r="A226" s="3" t="s">
         <x:v>483</x:v>
       </x:c>
-      <x:c r="K226" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="BC226" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="BZ226" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="CA226" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="CH226" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="CI226" s="6" t="s">
-        <x:v>129</x:v>
+      <x:c r="DI226" t="s">
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="227">
@@ -25709,7 +25862,22 @@
       <x:c r="B227" s="5" t="s">
         <x:v>485</x:v>
       </x:c>
-      <x:c r="BE227" s="6" t="s">
+      <x:c r="K227" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="BC227" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="BZ227" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="CA227" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="CH227" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="CI227" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
     </x:row>
@@ -25720,7 +25888,7 @@
       <x:c r="B228" s="5" t="s">
         <x:v>487</x:v>
       </x:c>
-      <x:c r="BR228" s="6" t="s">
+      <x:c r="BE228" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
     </x:row>
@@ -25731,7 +25899,7 @@
       <x:c r="B229" s="5" t="s">
         <x:v>489</x:v>
       </x:c>
-      <x:c r="X229" s="6" t="s">
+      <x:c r="BR229" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
     </x:row>
@@ -25740,23 +25908,20 @@
         <x:v>490</x:v>
       </x:c>
       <x:c r="B230" s="5" t="s">
-        <x:v>142</x:v>
-      </x:c>
-      <x:c r="CG230" s="6" t="s">
+        <x:v>491</x:v>
+      </x:c>
+      <x:c r="X230" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
     </x:row>
     <x:row r="231">
       <x:c r="A231" s="4" t="s">
-        <x:v>491</x:v>
+        <x:v>492</x:v>
       </x:c>
       <x:c r="B231" s="5" t="s">
-        <x:v>492</x:v>
-      </x:c>
-      <x:c r="D231" s="6" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="BJ231" s="6" t="s">
+        <x:v>142</x:v>
+      </x:c>
+      <x:c r="CG231" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
     </x:row>
@@ -25795,87 +25960,30 @@
       <x:c r="B234" s="5" t="s">
         <x:v>498</x:v>
       </x:c>
-      <x:c r="BK234" s="6" t="s">
+      <x:c r="D234" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="BJ234" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
     </x:row>
     <x:row r="235">
-      <x:c r="A235" s="3" t="s">
+      <x:c r="A235" s="4" t="s">
         <x:v>499</x:v>
       </x:c>
-      <x:c r="DI235" t="s">
-        <x:v>1</x:v>
+      <x:c r="B235" s="5" t="s">
+        <x:v>500</x:v>
+      </x:c>
+      <x:c r="BK235" s="6" t="s">
+        <x:v>129</x:v>
       </x:c>
     </x:row>
     <x:row r="236">
-      <x:c r="A236" s="4" t="s">
-        <x:v>500</x:v>
-      </x:c>
-      <x:c r="B236" s="5" t="s">
+      <x:c r="A236" s="3" t="s">
         <x:v>501</x:v>
       </x:c>
-      <x:c r="G236" s="8" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="I236" s="8" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="J236" s="8" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="L236" s="8" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="S236" s="8" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="T236" s="8" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="AT236" s="8" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="AU236" s="8" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="AV236" s="8" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="AW236" s="8" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="AX236" s="8" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="AZ236" s="8" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="BA236" s="8" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="BB236" s="8" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="BI236" s="8" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="BK236" s="8" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="CI236" s="8" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="CW236" s="8" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="DC236" s="8" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="DD236" s="8" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="DE236" s="8" t="s">
-        <x:v>129</x:v>
+      <x:c r="DI236" t="s">
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="237">
@@ -25885,66 +25993,24 @@
       <x:c r="B237" s="5" t="s">
         <x:v>503</x:v>
       </x:c>
-      <x:c r="E237" s="8" t="s">
-        <x:v>129</x:v>
-      </x:c>
       <x:c r="G237" s="8" t="s">
         <x:v>129</x:v>
       </x:c>
+      <x:c r="I237" s="8" t="s">
+        <x:v>129</x:v>
+      </x:c>
       <x:c r="J237" s="8" t="s">
         <x:v>129</x:v>
       </x:c>
       <x:c r="L237" s="8" t="s">
         <x:v>129</x:v>
       </x:c>
-      <x:c r="M237" s="8" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="N237" s="8" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="O237" s="8" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="P237" s="8" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="Q237" s="8" t="s">
-        <x:v>129</x:v>
-      </x:c>
       <x:c r="S237" s="8" t="s">
         <x:v>129</x:v>
       </x:c>
       <x:c r="T237" s="8" t="s">
         <x:v>129</x:v>
       </x:c>
-      <x:c r="U237" s="8" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="V237" s="8" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="W237" s="8" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="AB237" s="8" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="AC237" s="8" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="AD237" s="8" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="AE237" s="8" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="AF237" s="8" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="AG237" s="8" t="s">
-        <x:v>129</x:v>
-      </x:c>
       <x:c r="AT237" s="8" t="s">
         <x:v>129</x:v>
       </x:c>
@@ -25960,82 +26026,34 @@
       <x:c r="AX237" s="8" t="s">
         <x:v>129</x:v>
       </x:c>
-      <x:c r="AY237" s="8" t="s">
-        <x:v>129</x:v>
-      </x:c>
       <x:c r="AZ237" s="8" t="s">
         <x:v>129</x:v>
       </x:c>
-      <x:c r="BF237" s="8" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="BG237" s="8" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="BH237" s="8" t="s">
+      <x:c r="BA237" s="8" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="BB237" s="8" t="s">
         <x:v>129</x:v>
       </x:c>
       <x:c r="BI237" s="8" t="s">
         <x:v>129</x:v>
       </x:c>
-      <x:c r="BL237" s="8" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="BN237" s="8" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="BO237" s="8" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="BU237" s="8" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="CB237" s="8" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="CC237" s="8" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="CH237" s="8" t="s">
+      <x:c r="BK237" s="8" t="s">
         <x:v>129</x:v>
       </x:c>
       <x:c r="CI237" s="8" t="s">
         <x:v>129</x:v>
       </x:c>
-      <x:c r="CP237" s="8" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="CU237" s="8" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="CV237" s="8" t="s">
-        <x:v>129</x:v>
-      </x:c>
       <x:c r="CW237" s="8" t="s">
         <x:v>129</x:v>
       </x:c>
-      <x:c r="CX237" s="8" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="CY237" s="8" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="DA237" s="8" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="DB237" s="8" t="s">
+      <x:c r="DC237" s="8" t="s">
         <x:v>129</x:v>
       </x:c>
       <x:c r="DD237" s="8" t="s">
         <x:v>129</x:v>
       </x:c>
       <x:c r="DE237" s="8" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="DH237" s="8" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="DI237" s="8" t="s">
         <x:v>129</x:v>
       </x:c>
     </x:row>
@@ -26046,19 +26064,16 @@
       <x:c r="B238" s="5" t="s">
         <x:v>505</x:v>
       </x:c>
-      <x:c r="C238" s="8" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="D238" s="8" t="s">
-        <x:v>129</x:v>
-      </x:c>
       <x:c r="E238" s="8" t="s">
         <x:v>129</x:v>
       </x:c>
-      <x:c r="F238" s="8" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="K238" s="8" t="s">
+      <x:c r="G238" s="8" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="J238" s="8" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="L238" s="8" t="s">
         <x:v>129</x:v>
       </x:c>
       <x:c r="M238" s="8" t="s">
@@ -26076,24 +26091,21 @@
       <x:c r="Q238" s="8" t="s">
         <x:v>129</x:v>
       </x:c>
+      <x:c r="S238" s="8" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="T238" s="8" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="U238" s="8" t="s">
+        <x:v>129</x:v>
+      </x:c>
       <x:c r="V238" s="8" t="s">
         <x:v>129</x:v>
       </x:c>
       <x:c r="W238" s="8" t="s">
         <x:v>129</x:v>
       </x:c>
-      <x:c r="X238" s="8" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="Y238" s="8" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="Z238" s="8" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="AA238" s="8" t="s">
-        <x:v>129</x:v>
-      </x:c>
       <x:c r="AB238" s="8" t="s">
         <x:v>129</x:v>
       </x:c>
@@ -26112,55 +26124,25 @@
       <x:c r="AG238" s="8" t="s">
         <x:v>129</x:v>
       </x:c>
-      <x:c r="AH238" s="8" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="AI238" s="8" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="AJ238" s="8" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="AK238" s="8" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="AL238" s="8" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="AM238" s="8" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="AN238" s="8" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="AO238" s="8" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="AP238" s="8" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="AQ238" s="8" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="AR238" s="8" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="AS238" s="8" t="s">
+      <x:c r="AT238" s="8" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="AU238" s="8" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="AV238" s="8" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="AW238" s="8" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="AX238" s="8" t="s">
         <x:v>129</x:v>
       </x:c>
       <x:c r="AY238" s="8" t="s">
         <x:v>129</x:v>
       </x:c>
-      <x:c r="BA238" s="8" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="BB238" s="8" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="BC238" s="8" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="BD238" s="8" t="s">
+      <x:c r="AZ238" s="8" t="s">
         <x:v>129</x:v>
       </x:c>
       <x:c r="BF238" s="8" t="s">
@@ -26172,7 +26154,7 @@
       <x:c r="BH238" s="8" t="s">
         <x:v>129</x:v>
       </x:c>
-      <x:c r="BJ238" s="8" t="s">
+      <x:c r="BI238" s="8" t="s">
         <x:v>129</x:v>
       </x:c>
       <x:c r="BL238" s="8" t="s">
@@ -26184,43 +26166,13 @@
       <x:c r="BO238" s="8" t="s">
         <x:v>129</x:v>
       </x:c>
-      <x:c r="BQ238" s="8" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="BR238" s="8" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="BS238" s="8" t="s">
-        <x:v>129</x:v>
-      </x:c>
       <x:c r="BU238" s="8" t="s">
         <x:v>129</x:v>
       </x:c>
-      <x:c r="BW238" s="8" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="BX238" s="8" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="BY238" s="8" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="BZ238" s="8" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="CA238" s="8" t="s">
-        <x:v>129</x:v>
-      </x:c>
       <x:c r="CB238" s="8" t="s">
         <x:v>129</x:v>
       </x:c>
-      <x:c r="CD238" s="8" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="CF238" s="8" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="CG238" s="8" t="s">
+      <x:c r="CC238" s="8" t="s">
         <x:v>129</x:v>
       </x:c>
       <x:c r="CH238" s="8" t="s">
@@ -26229,55 +26181,34 @@
       <x:c r="CI238" s="8" t="s">
         <x:v>129</x:v>
       </x:c>
-      <x:c r="CJ238" s="8" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="CK238" s="8" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="CL238" s="8" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="CM238" s="8" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="CO238" s="8" t="s">
-        <x:v>129</x:v>
-      </x:c>
       <x:c r="CP238" s="8" t="s">
         <x:v>129</x:v>
       </x:c>
-      <x:c r="CQ238" s="8" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="CS238" s="8" t="s">
-        <x:v>129</x:v>
-      </x:c>
       <x:c r="CU238" s="8" t="s">
         <x:v>129</x:v>
       </x:c>
       <x:c r="CV238" s="8" t="s">
         <x:v>129</x:v>
       </x:c>
+      <x:c r="CW238" s="8" t="s">
+        <x:v>129</x:v>
+      </x:c>
       <x:c r="CX238" s="8" t="s">
         <x:v>129</x:v>
       </x:c>
       <x:c r="CY238" s="8" t="s">
         <x:v>129</x:v>
       </x:c>
-      <x:c r="CZ238" s="8" t="s">
-        <x:v>129</x:v>
-      </x:c>
       <x:c r="DA238" s="8" t="s">
         <x:v>129</x:v>
       </x:c>
       <x:c r="DB238" s="8" t="s">
         <x:v>129</x:v>
       </x:c>
-      <x:c r="DC238" s="8" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="DF238" s="8" t="s">
+      <x:c r="DD238" s="8" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="DE238" s="8" t="s">
         <x:v>129</x:v>
       </x:c>
       <x:c r="DH238" s="8" t="s">
@@ -26288,343 +26219,591 @@
       </x:c>
     </x:row>
     <x:row r="239">
-      <x:c r="A239" s="9" t="s">
+      <x:c r="A239" s="4" t="s">
+        <x:v>506</x:v>
+      </x:c>
+      <x:c r="B239" s="5" t="s">
+        <x:v>507</x:v>
+      </x:c>
+      <x:c r="C239" s="8" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="D239" s="8" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="E239" s="8" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="F239" s="8" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="K239" s="8" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="M239" s="8" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="N239" s="8" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="O239" s="8" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="P239" s="8" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="Q239" s="8" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="V239" s="8" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="W239" s="8" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="X239" s="8" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="Y239" s="8" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="Z239" s="8" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="AA239" s="8" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="AB239" s="8" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="AC239" s="8" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="AD239" s="8" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="AE239" s="8" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="AF239" s="8" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="AG239" s="8" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="AH239" s="8" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="AI239" s="8" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="AJ239" s="8" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="AK239" s="8" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="AL239" s="8" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="AM239" s="8" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="AN239" s="8" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="AO239" s="8" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="AP239" s="8" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="AQ239" s="8" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="AR239" s="8" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="AS239" s="8" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="AY239" s="8" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="BA239" s="8" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="BB239" s="8" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="BC239" s="8" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="BD239" s="8" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="BF239" s="8" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="BG239" s="8" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="BH239" s="8" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="BJ239" s="8" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="BL239" s="8" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="BN239" s="8" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="BO239" s="8" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="BQ239" s="8" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="BR239" s="8" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="BS239" s="8" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="BU239" s="8" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="BW239" s="8" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="BX239" s="8" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="BY239" s="8" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="BZ239" s="8" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="CA239" s="8" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="CB239" s="8" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="CD239" s="8" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="CF239" s="8" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="CG239" s="8" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="CH239" s="8" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="CI239" s="8" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="CJ239" s="8" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="CK239" s="8" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="CL239" s="8" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="CM239" s="8" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="CO239" s="8" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="CP239" s="8" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="CQ239" s="8" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="CS239" s="8" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="CU239" s="8" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="CV239" s="8" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="CX239" s="8" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="CY239" s="8" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="CZ239" s="8" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="DA239" s="8" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="DB239" s="8" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="DC239" s="8" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="DF239" s="8" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="DH239" s="8" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="DI239" s="8" t="s">
+        <x:v>129</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="240">
+      <x:c r="A240" s="9" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="B239" s="9" t="s">
+      <x:c r="B240" s="9" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="C239" s="9" t="s">
+      <x:c r="C240" s="9" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="D239" s="9" t="s">
+      <x:c r="D240" s="9" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="E239" s="9" t="s">
+      <x:c r="E240" s="9" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="F239" s="9" t="s">
+      <x:c r="F240" s="9" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="G239" s="9" t="s">
+      <x:c r="G240" s="9" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H239" s="9" t="s">
+      <x:c r="H240" s="9" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="I239" s="9" t="s">
+      <x:c r="I240" s="9" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="J239" s="9" t="s">
+      <x:c r="J240" s="9" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="K239" s="9" t="s">
+      <x:c r="K240" s="9" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="L239" s="9" t="s">
+      <x:c r="L240" s="9" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="M239" s="9" t="s">
+      <x:c r="M240" s="9" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="N239" s="9" t="s">
+      <x:c r="N240" s="9" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="O239" s="9" t="s">
+      <x:c r="O240" s="9" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="P239" s="9" t="s">
+      <x:c r="P240" s="9" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="Q239" s="9" t="s">
+      <x:c r="Q240" s="9" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="R239" s="9" t="s">
+      <x:c r="R240" s="9" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="S239" s="9" t="s">
+      <x:c r="S240" s="9" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="T239" s="9" t="s">
+      <x:c r="T240" s="9" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="U239" s="9" t="s">
+      <x:c r="U240" s="9" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="V239" s="9" t="s">
+      <x:c r="V240" s="9" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="W239" s="9" t="s">
+      <x:c r="W240" s="9" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="X239" s="9" t="s">
+      <x:c r="X240" s="9" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="Y239" s="9" t="s">
+      <x:c r="Y240" s="9" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="Z239" s="9" t="s">
+      <x:c r="Z240" s="9" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="AA239" s="9" t="s">
+      <x:c r="AA240" s="9" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="AB239" s="9" t="s">
+      <x:c r="AB240" s="9" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="AC239" s="9" t="s">
+      <x:c r="AC240" s="9" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="AD239" s="9" t="s">
+      <x:c r="AD240" s="9" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="AE239" s="9" t="s">
+      <x:c r="AE240" s="9" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="AF239" s="9" t="s">
+      <x:c r="AF240" s="9" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="AG239" s="9" t="s">
+      <x:c r="AG240" s="9" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="AH239" s="9" t="s">
+      <x:c r="AH240" s="9" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="AI239" s="9" t="s">
+      <x:c r="AI240" s="9" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="AJ239" s="9" t="s">
+      <x:c r="AJ240" s="9" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="AK239" s="9" t="s">
+      <x:c r="AK240" s="9" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="AL239" s="9" t="s">
+      <x:c r="AL240" s="9" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="AM239" s="9" t="s">
+      <x:c r="AM240" s="9" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="AN239" s="9" t="s">
+      <x:c r="AN240" s="9" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="AO239" s="9" t="s">
+      <x:c r="AO240" s="9" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="AP239" s="9" t="s">
+      <x:c r="AP240" s="9" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="AQ239" s="9" t="s">
+      <x:c r="AQ240" s="9" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="AR239" s="9" t="s">
+      <x:c r="AR240" s="9" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="AS239" s="9" t="s">
+      <x:c r="AS240" s="9" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="AT239" s="9" t="s">
+      <x:c r="AT240" s="9" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="AU239" s="9" t="s">
+      <x:c r="AU240" s="9" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="AV239" s="9" t="s">
+      <x:c r="AV240" s="9" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="AW239" s="9" t="s">
+      <x:c r="AW240" s="9" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="AX239" s="9" t="s">
+      <x:c r="AX240" s="9" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="AY239" s="9" t="s">
+      <x:c r="AY240" s="9" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="AZ239" s="9" t="s">
+      <x:c r="AZ240" s="9" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="BA239" s="9" t="s">
+      <x:c r="BA240" s="9" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="BB239" s="9" t="s">
+      <x:c r="BB240" s="9" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="BC239" s="9" t="s">
+      <x:c r="BC240" s="9" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="BD239" s="9" t="s">
+      <x:c r="BD240" s="9" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="BE239" s="9" t="s">
+      <x:c r="BE240" s="9" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="BF239" s="9" t="s">
+      <x:c r="BF240" s="9" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="BG239" s="9" t="s">
+      <x:c r="BG240" s="9" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="BH239" s="9" t="s">
+      <x:c r="BH240" s="9" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="BI239" s="9" t="s">
+      <x:c r="BI240" s="9" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="BJ239" s="9" t="s">
+      <x:c r="BJ240" s="9" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="BK239" s="9" t="s">
+      <x:c r="BK240" s="9" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="BL239" s="9" t="s">
+      <x:c r="BL240" s="9" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="BM239" s="9" t="s">
+      <x:c r="BM240" s="9" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="BN239" s="9" t="s">
+      <x:c r="BN240" s="9" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="BO239" s="9" t="s">
+      <x:c r="BO240" s="9" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="BP239" s="9" t="s">
+      <x:c r="BP240" s="9" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="BQ239" s="9" t="s">
+      <x:c r="BQ240" s="9" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="BR239" s="9" t="s">
+      <x:c r="BR240" s="9" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="BS239" s="9" t="s">
+      <x:c r="BS240" s="9" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="BT239" s="9" t="s">
+      <x:c r="BT240" s="9" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="BU239" s="9" t="s">
+      <x:c r="BU240" s="9" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="BV239" s="9" t="s">
+      <x:c r="BV240" s="9" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="BW239" s="9" t="s">
+      <x:c r="BW240" s="9" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="BX239" s="9" t="s">
+      <x:c r="BX240" s="9" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="BY239" s="9" t="s">
+      <x:c r="BY240" s="9" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="BZ239" s="9" t="s">
+      <x:c r="BZ240" s="9" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="CA239" s="9" t="s">
+      <x:c r="CA240" s="9" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="CB239" s="9" t="s">
+      <x:c r="CB240" s="9" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="CC239" s="9" t="s">
+      <x:c r="CC240" s="9" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="CD239" s="9" t="s">
+      <x:c r="CD240" s="9" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="CE239" s="9" t="s">
+      <x:c r="CE240" s="9" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="CF239" s="9" t="s">
+      <x:c r="CF240" s="9" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="CG239" s="9" t="s">
+      <x:c r="CG240" s="9" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="CH239" s="9" t="s">
+      <x:c r="CH240" s="9" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="CI239" s="9" t="s">
+      <x:c r="CI240" s="9" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="CJ239" s="9" t="s">
+      <x:c r="CJ240" s="9" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="CK239" s="9" t="s">
+      <x:c r="CK240" s="9" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="CL239" s="9" t="s">
+      <x:c r="CL240" s="9" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="CM239" s="9" t="s">
+      <x:c r="CM240" s="9" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="CN239" s="9" t="s">
+      <x:c r="CN240" s="9" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="CO239" s="9" t="s">
+      <x:c r="CO240" s="9" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="CP239" s="9" t="s">
+      <x:c r="CP240" s="9" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="CQ239" s="9" t="s">
+      <x:c r="CQ240" s="9" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="CR239" s="9" t="s">
+      <x:c r="CR240" s="9" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="CS239" s="9" t="s">
+      <x:c r="CS240" s="9" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="CT239" s="9" t="s">
+      <x:c r="CT240" s="9" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="CU239" s="9" t="s">
+      <x:c r="CU240" s="9" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="CV239" s="9" t="s">
+      <x:c r="CV240" s="9" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="CW239" s="9" t="s">
+      <x:c r="CW240" s="9" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="CX239" s="9" t="s">
+      <x:c r="CX240" s="9" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="CY239" s="9" t="s">
+      <x:c r="CY240" s="9" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="CZ239" s="9" t="s">
+      <x:c r="CZ240" s="9" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="DA239" s="9" t="s">
+      <x:c r="DA240" s="9" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="DB239" s="9" t="s">
+      <x:c r="DB240" s="9" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="DC239" s="9" t="s">
+      <x:c r="DC240" s="9" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="DD239" s="9" t="s">
+      <x:c r="DD240" s="9" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="DE239" s="9" t="s">
+      <x:c r="DE240" s="9" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="DF239" s="9" t="s">
+      <x:c r="DF240" s="9" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="DG239" s="9" t="s">
+      <x:c r="DG240" s="9" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="DH239" s="9" t="s">
+      <x:c r="DH240" s="9" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="DI239" s="9" t="s">
+      <x:c r="DI240" s="9" t="s">
         <x:v>1</x:v>
       </x:c>
     </x:row>
@@ -26675,8 +26854,8 @@
     <x:mergeCell ref="A189:DI189"/>
     <x:mergeCell ref="A196:DI196"/>
     <x:mergeCell ref="A207:DI207"/>
-    <x:mergeCell ref="A225:DI225"/>
-    <x:mergeCell ref="A235:DI235"/>
+    <x:mergeCell ref="A226:DI226"/>
+    <x:mergeCell ref="A236:DI236"/>
   </x:mergeCells>
 </x:worksheet>
 </file>
</xml_diff>